<commit_message>
test github STchatGPT access
</commit_message>
<xml_diff>
--- a/datasets/07_delivery/st_ready/quality_test_suite_all_series.xlsx
+++ b/datasets/07_delivery/st_ready/quality_test_suite_all_series.xlsx
@@ -1,29 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stmicroelectronics-my.sharepoint.com/personal/abir_gharbi_st_com/Documents/Desktop/PFE_Chatbot_STM32Cube/datasets/07_delivery/st_ready/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_C8F10CE654659E7FE01694954D5DCE3A8743D547" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A2A08CD6-A984-4597-B36C-49784B55C274}"/>
+  <xr:revisionPtr revIDLastSave="24" documentId="11_C8F10CE654659E7FE01694954D5DCE3A8743D547" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{39B98395-2EBC-462C-9D72-8CEA4820FD19}"/>
   <bookViews>
-    <workbookView xWindow="-25320" yWindow="-21720" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Quality Test Suite" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Quality Test Suite'!$A$1:$C$97</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Quality Test Suite'!$A$1:$C$71</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="166">
   <si>
     <t>Question</t>
   </si>
@@ -252,144 +252,6 @@
 4. **Test with a minimal project**
 5. **Add custom code back incrementally**
 If you want, I can also provide a **peripheral-init migration checklist template** for a specific STM32H7 peripheral such as **USART, SPI, I2C, ADC, ETH, USB, FMC, or SDMMC**.</t>
-  </si>
-  <si>
-    <t>On STM32CubeH7, I2C sometimes gets stuck BUSY after a communication error and the bus never recovers. What is a safe software recovery sequence without full MCU reset?</t>
-  </si>
-  <si>
-    <t>Here is a **safe software recovery sequence** for an **STM32H7 I2C peripheral** that remains **BUSY** after a communication error.
-## Goal
-Recover the I2C bus **without resetting the full MCU**, by:
-1. **Stopping the I2C peripheral**
-2. **Forcing the bus lines free**
-3. **Reinitializing the peripheral**
-4. **Restarting communication cleanly**
----
-## Recommended recovery sequence
-### 1) Disable the I2C peripheral
-Abort any ongoing transfer and stop the peripheral:
-```c
-__HAL_I2C_DISABLE(&amp;hi2c1);
-```
-If you use interrupts/DMA, also stop them first:
-- disable I2C interrupts
-- abort DMA if active
-- clear pending flags in software
----
-### 2) Put I2C pins in GPIO open-drain mode
-Reconfigure **SCL** and **SDA** as **GPIO open-drain outputs** with pull-up enabled, so you can manually clock the bus.
-```c
-GPIO_InitTypeDef GPIO_InitStruct = {0};
-GPIO_InitStruct.Pin = I2C1_SCL_Pin | I2C1_SDA_Pin;
-GPIO_InitStruct.Mode = GPIO_MODE_OUTPUT_OD;
-GPIO_InitStruct.Pull = GPIO_PULLUP;
-GPIO_InitStruct.Speed = GPIO_SPEED_FREQ_HIGH;
-HAL_GPIO_Init(I2C1_GPIO_Port, &amp;GPIO_InitStruct);
-```
----
-### 3) Release SDA and toggle SCL until SDA is released
-If a slave is holding SDA low, generate up to **9 clock pulses** on SCL to let the slave complete its internal state machine.
-```c
-for (int i = 0; i &lt; 9; i++)
-{
-    HAL_GPIO_WritePin(I2C1_GPIO_Port, I2C1_SCL_Pin, GPIO_PIN_RESET);
-    delay_us(5);
-    HAL_GPIO_WritePin(I2C1_GPIO_Port, I2C1_SCL_Pin, GPIO_PIN_SET);
-    delay_us(5);
-    if (HAL_GPIO_ReadPin(I2C1_GPIO_Port, I2C1_SDA_Pin) == GPIO_PIN_SET)
-        break;
-}
-```
----
-### 4) Generate a STOP condition manually
-Once SDA is released, create a STOP condition:
-- SCL high
-- SDA transition low → high while SCL is high
-```c
-HAL_GPIO_WritePin(I2C1_GPIO_Port, I2C1_SDA_Pin, GPIO_PIN_RESET);
-delay_us(5);
-HAL_GPIO_WritePin(I2C1_GPIO_Port, I2C1_SCL_Pin, GPIO_PIN_SET);
-delay_us(5);
-HAL_GPIO_WritePin(I2C1_GPIO_Port, I2C1_SDA_Pin, GPIO_PIN_SET);
-delay_us(5);
-```
----
-### 5) Restore the peripheral pins to I2C alternate function
-Return SCL/SDA to their I2C AF configuration.
-```c
-HAL_GPIO_Init(I2C1_GPIO_Port, &amp;GPIO_InitStruct_AF);
-```
----
-### 6) Reinitialize the I2C peripheral
-Clear internal state and reinitialize:
-```c
-HAL_I2C_DeInit(&amp;hi2c1);
-HAL_I2C_Init(&amp;hi2c1);
-```
-If needed, also reconfigure timing and filters via CubeMX-generated init code.
----
-## Strongly recommended: add peripheral reset if GPIO recovery fails
-If the bus is still stuck after GPIO clocking, perform a **peripheral reset only**:
-```c
-__HAL_RCC_I2C1_FORCE_RESET();
-__HAL_RCC_I2C1_RELEASE_RESET();
-```
-Then reinitialize I2C again.
-This is usually safer and faster than a full system reset.
----
-## Minimal robust recovery function
-```c
-void I2C1_BusRecover(void)
-{
-    GPIO_InitTypeDef GPIO_InitStruct = {0};
-    // 1. Disable I2C
-    __HAL_I2C_DISABLE(&amp;hi2c1);
-    // 2. Configure pins as GPIO open-drain
-    GPIO_InitStruct.Pin = I2C1_SCL_Pin | I2C1_SDA_Pin;
-    GPIO_InitStruct.Mode = GPIO_MODE_OUTPUT_OD;
-    GPIO_InitStruct.Pull = GPIO_PULLUP;
-    GPIO_InitStruct.Speed = GPIO_SPEED_FREQ_HIGH;
-    HAL_GPIO_Init(I2C1_GPIO_Port, &amp;GPIO_InitStruct);
-    // 3. Try to free SDA by clocking SCL
-    HAL_GPIO_WritePin(I2C1_GPIO_Port, I2C1_SCL_Pin, GPIO_PIN_SET);
-    HAL_GPIO_WritePin(I2C1_GPIO_Port, I2C1_SDA_Pin, GPIO_PIN_SET);
-    HAL_Delay(1);
-    for (int i = 0; i &lt; 9; i++)
-    {
-        HAL_GPIO_WritePin(I2C1_GPIO_Port, I2C1_SCL_Pin, GPIO_PIN_RESET);
-        delay_us(5);
-        HAL_GPIO_WritePin(I2C1_GPIO_Port, I2C1_SCL_Pin, GPIO_PIN_SET);
-        delay_us(5);
-        if (HAL_GPIO_ReadPin(I2C1_GPIO_Port, I2C1_SDA_Pin) == GPIO_PIN_SET)
-            break;
-    }
-    // 4. Generate STOP
-    HAL_GPIO_WritePin(I2C1_GPIO_Port, I2C1_SDA_Pin, GPIO_PIN_RESET);
-    delay_us(5);
-    HAL_GPIO_WritePin(I2C1_GPIO_Port, I2C1_SCL_Pin, GPIO_PIN_SET);
-    delay_us(5);
-    HAL_GPIO_WritePin(I2C1_GPIO_Port, I2C1_SDA_Pin, GPIO_PIN_SET);
-    delay_us(5);
-    // 5. Restore AF pins
-    HAL_GPIO_Init(I2C1_GPIO_Port, &amp;GPIO_InitStruct_AF);
-    // 6. Reset and reinit peripheral
-    HAL_I2C_DeInit(&amp;hi2c1);
-    HAL_I2C_Init(&amp;hi2c1);
-}
-```
----
-## Notes specific to STM32H7
-- If **D-cache**, **DMA**, or **interrupt-driven transfers** are involved, make sure the transaction is fully aborted before reinitializing.
-- If your I2C uses **analog or digital filters**, keep the same timing/filter configuration after recovery.
-- If the bus is externally held low by a damaged slave or missing pull-up, software recovery will not succeed.
----
-## Best practice
-Also add:
-- **Timeouts** on every transaction
-- **Error callback** recovery path
-- Optional **bus-clear watchdog** logic
-- A **fallback peripheral reset** after failed GPIO recovery
-If you want, I can provide a **CubeH7/HAL-ready recovery function** tailored to your exact I2C instance and pin names.</t>
   </si>
   <si>
     <t>I need lower power consumption on STM32CubeH7 while preserving wake-up reliability. Which low-power configuration points should be audited first (clocks, GPIO state, peripherals, wake-up sources)?</t>
@@ -694,138 +556,6 @@
 If you want, I can turn this into a **one-page migration checklist template** you can reuse for any STM32Cube package update.</t>
   </si>
   <si>
-    <t>On STM32CubeC0, I2C sometimes gets stuck BUSY after a communication error and the bus never recovers. What is a safe software recovery sequence without full MCU reset?</t>
-  </si>
-  <si>
-    <t>A safe software recovery for a **stuck I2C BUSY** condition on **STM32CubeC0** is typically:
-1. **Stop the I2C peripheral**
-2. **Disable I2C**
-3. **Release the bus lines by switching SCL/SDA to GPIO open-drain**
-4. **Manually generate clock pulses on SCL** to free a slave holding SDA low
-5. **Optionally generate a STOP condition**
-6. **Reinitialize the peripheral**
-7. **Retry the transfer**
-## Recommended recovery sequence
-### 1) Abort any ongoing transfer
-If using HAL, first abort the peripheral transaction if possible:
-```c
-HAL_I2C_Master_Abort_IT(&amp;hi2c1, addr);
-```
-If the bus is already wedged, you may need to move directly to peripheral disable/recovery.
----
-### 2) Disable I2C peripheral
-Disable the peripheral so the GPIOs can be controlled manually:
-```c
-__HAL_I2C_DISABLE(&amp;hi2c1);
-```
-If needed, also disable I2C interrupts and DMA channels.
----
-### 3) Reconfigure SCL and SDA as GPIO open-drain
-Switch both pins to **GPIO output open-drain with pull-up** or use external pull-ups if available.
-Typical setup:
-- SCL: output open-drain
-- SDA: output open-drain
-- Drive high by releasing the line
-- Drive low only when needed
----
-### 4) Generate up to 9 SCL pulses
-A slave may be holding SDA low waiting for more clocks. Toggle SCL about 9 times while monitoring SDA.
-Pseudo-code:
-```c
-for (int i = 0; i &lt; 9; i++)
-{
-    HAL_GPIO_WritePin(SCL_GPIO_Port, SCL_Pin, GPIO_PIN_RESET);
-    delay_us(5);
-    HAL_GPIO_WritePin(SCL_GPIO_Port, SCL_Pin, GPIO_PIN_SET);
-    delay_us(5);
-    if (HAL_GPIO_ReadPin(SDA_GPIO_Port, SDA_Pin) == GPIO_PIN_SET)
-        break;
-}
-```
-If SDA is released before 9 pulses, the bus is likely recovered.
----
-### 5) Force a STOP condition
-With SCL high, transition SDA from low to high:
-```c
-HAL_GPIO_WritePin(SDA_GPIO_Port, SDA_Pin, GPIO_PIN_RESET);
-delay_us(5);
-HAL_GPIO_WritePin(SCL_GPIO_Port, SCL_Pin, GPIO_PIN_SET);
-delay_us(5);
-HAL_GPIO_WritePin(SDA_GPIO_Port, SDA_Pin, GPIO_PIN_SET);
-delay_us(5);
-```
-This is only meaningful if the lines are under GPIO control and are actually being released high by pull-ups.
----
-### 6) Restore I2C alternate function
-Return SCL/SDA to I2C AF mode and reinitialize:
-```c
-HAL_I2C_Init(&amp;hi2c1);
-```
-If you use CubeMX-generated init, you may need to call the MSP init or deinit/init sequence depending on your project structure.
----
-## Practical safe implementation pattern
-A robust recovery function looks like this:
-```c
-HAL_StatusTypeDef I2C_Recover(I2C_HandleTypeDef *hi2c)
-{
-    GPIO_InitTypeDef GPIO_InitStruct = {0};
-    __HAL_I2C_DISABLE(hi2c);
-    // Deinit I2C GPIOs from AF mode
-    HAL_GPIO_DeInit(SCL_GPIO_Port, SCL_Pin);
-    HAL_GPIO_DeInit(SDA_GPIO_Port, SDA_Pin);
-    // Configure as GPIO OD
-    GPIO_InitStruct.Pin = SCL_Pin | SDA_Pin;
-    GPIO_InitStruct.Mode = GPIO_MODE_OUTPUT_OD;
-    GPIO_InitStruct.Pull = GPIO_PULLUP;
-    GPIO_InitStruct.Speed = GPIO_SPEED_FREQ_LOW;
-    HAL_GPIO_Init(GPIO_Port, &amp;GPIO_InitStruct);
-    // Release both lines
-    HAL_GPIO_WritePin(GPIO_Port, SCL_Pin | SDA_Pin, GPIO_PIN_SET);
-    delay_us(5);
-    // Clock out stuck slave
-    for (int i = 0; i &lt; 9; i++)
-    {
-        HAL_GPIO_WritePin(GPIO_Port, SCL_Pin, GPIO_PIN_RESET);
-        delay_us(5);
-        HAL_GPIO_WritePin(GPIO_Port, SCL_Pin, GPIO_PIN_SET);
-        delay_us(5);
-        if (HAL_GPIO_ReadPin(GPIO_Port, SDA_Pin) == GPIO_PIN_SET)
-            break;
-    }
-    // Generate STOP
-    HAL_GPIO_WritePin(GPIO_Port, SDA_Pin, GPIO_PIN_LOW);
-    delay_us(5);
-    HAL_GPIO_WritePin(GPIO_Port, SCL_Pin, GPIO_PIN_SET);
-    delay_us(5);
-    HAL_GPIO_WritePin(GPIO_Port, SDA_Pin, GPIO_PIN_SET);
-    delay_us(5);
-    // Restore AF mode / reinit I2C
-    HAL_GPIO_DeInit(GPIO_Port, SCL_Pin | SDA_Pin);
-    MX_I2C1_Init();   // or HAL_I2C_Init(hi2c)
-    return HAL_OK;
-}
-```
----
-## Important notes
-- **Do not rely on just clearing error flags** if BUSY stays set; that usually means the bus lines are physically stuck.
-- If **SDA is held low by the peripheral itself** due to an internal state machine issue, the safest fix is:
-  - disable I2C,
-  - reconfigure pins to GPIO,
-  - pulse SCL,
-  - reinit peripheral.
-- If hardware pull-ups are weak or missing, recovery may fail.
-- Add a **timeout** around any I2C transaction so recovery is triggered automatically.
----
-## Best practice
-For STM32CubeC0, the safest production approach is:
-- detect I2C timeout/error,
-- call a **bus recovery routine**,
-- reinitialize I2C,
-- retry once,
-- if it still fails, flag the device as degraded and log the fault.
-If you want, I can provide a **CubeMX-ready C recovery function** tailored to your exact **I2C instance and pin names**.</t>
-  </si>
-  <si>
     <t>I need lower power consumption on STM32CubeC0 while preserving wake-up reliability. Which low-power configuration points should be audited first (clocks, GPIO state, peripherals, wake-up sources)?</t>
   </si>
   <si>
@@ -1194,101 +924,6 @@
 - `HAL_RCC_GetPCLK1Freq()`
 ---
 If you want, I can also provide a **one-page STM32CubeF0 migration checklist template** you can use directly during updates.</t>
-  </si>
-  <si>
-    <t>On STM32CubeF0, I2C sometimes gets stuck BUSY after a communication error and the bus never recovers. What is a safe software recovery sequence without full MCU reset?</t>
-  </si>
-  <si>
-    <t>A safe STM32CubeF0 software recovery sequence for a wedged I2C bus is:
-## 1) Stop the peripheral cleanly
-- Disable the I2C peripheral
-- Clear any pending error/stop flags
-- Abort any ongoing transfer if your code uses interrupts/DMA
-## 2) Release the bus in GPIO mode
-Reconfigure:
-- **SCL** as **GPIO open-drain output**
-- **SDA** as **GPIO open-drain input/output** with pull-up enabled
-Then manually generate **up to 9 SCL pulses** while monitoring SDA.
-### Why 9 pulses?
-A slave may be holding SDA low waiting for clock edges to finish an incomplete byte. Nine clocks is the standard recovery to flush one stuck byte plus ACK phase.
-## 3) Generate a STOP condition manually
-If SDA is released high after the clock pulses:
-- Drive **SDA low**
-- Drive **SCL high**
-- Release **SDA high**
-This creates a valid STOP and helps reset slave state machines.
-## 4) Reinitialize the I2C peripheral
-- Restore the I2C pin AF configuration
-- Re-enable the I2C peripheral
-- Reconfigure timing / own address / filters as needed
-- Clear error flags again before restarting communication
----
-# Recommended sequence in code terms
-## Recovery flow
-1. `__HAL_I2C_DISABLE(hi2c)`
-2. Abort DMA/IT if used
-3. Deinit I2C pins from AF mode
-4. Configure SCL/SDA as GPIO open-drain with pull-up
-5. If **SDA = 0**, toggle **SCL** 9 times:
-   - `SCL low`
-   - short delay
-   - `SCL high`
-   - short delay
-   - stop early if SDA goes high
-6. Generate STOP:
-   - `SDA low`
-   - `SCL high`
-   - `SDA high`
-7. Reconfigure pins back to I2C AF
-8. Clear I2C error/status
-9. `__HAL_I2C_ENABLE(hi2c)`
----
-# Practical notes for STM32F0
-- If the line is held low by a **powered-off slave**, clocking won’t help until the slave is powered or isolated.
-- If **SCL is low**, a slave or external hardware is actively stretching or faulting; software recovery may not be possible.
-- Use **timeouts** around every transfer, and on timeout call the recovery routine before retrying.
-- After recovery, it is often best to **recreate the I2C handle state** rather than only clearing flags.
----
-# Minimal recovery template
-```c
-static void I2C_BusRecover(I2C_HandleTypeDef *hi2c)
-{
-    GPIO_InitTypeDef GPIO_InitStruct = {0};
-    __HAL_I2C_DISABLE(hi2c);
-    HAL_I2C_DeInit(hi2c);
-    // Configure SCL/SDA as GPIO open-drain with pull-up
-    GPIO_InitStruct.Mode  = GPIO_MODE_OUTPUT_OD;
-    GPIO_InitStruct.Pull  = GPIO_PULLUP;
-    GPIO_InitStruct.Speed = GPIO_SPEED_FREQ_LOW;
-    GPIO_InitStruct.Pin = I2C_SCL_PIN;
-    HAL_GPIO_Init(I2C_SCL_GPIO_PORT, &amp;GPIO_InitStruct);
-    GPIO_InitStruct.Pin = I2C_SDA_PIN;
-    HAL_GPIO_Init(I2C_SDA_GPIO_PORT, &amp;GPIO_InitStruct);
-    // If SDA is low, toggle SCL up to 9 times
-    for (int i = 0; i &lt; 9 &amp;&amp; HAL_GPIO_ReadPin(I2C_SDA_GPIO_PORT, I2C_SDA_PIN) == GPIO_PIN_RESET; i++)
-    {
-        HAL_GPIO_WritePin(I2C_SCL_GPIO_PORT, I2C_SCL_PIN, GPIO_PIN_RESET);
-        HAL_Delay(1);
-        HAL_GPIO_WritePin(I2C_SCL_GPIO_PORT, I2C_SCL_PIN, GPIO_PIN_SET);
-        HAL_Delay(1);
-    }
-    // Generate STOP
-    HAL_GPIO_WritePin(I2C_SDA_GPIO_PORT, I2C_SDA_PIN, GPIO_PIN_RESET);
-    HAL_Delay(1);
-    HAL_GPIO_WritePin(I2C_SCL_GPIO_PORT, I2C_SCL_PIN, GPIO_PIN_SET);
-    HAL_Delay(1);
-    HAL_GPIO_WritePin(I2C_SDA_GPIO_PORT, I2C_SDA_PIN, GPIO_PIN_SET);
-    HAL_Delay(1);
-    // Restore AF mode is board-specific; reinit I2C afterwards
-    HAL_I2C_Init(hi2c);
-}
-```
----
-# Important caveats
-- On STM32F0, make sure the GPIOs are on a port/pin pair that can be safely reconfigured at runtime.
-- If the bus is shared with other masters, coordinate recovery carefully.
-- If the peripheral is stuck due to a **hardware erratum or bus contention**, the only reliable fix may be removing the fault source.
-If you want, I can provide a **CubeMX-compatible recovery function for a specific STM32F0 part number and I2C instance**.</t>
   </si>
   <si>
     <t>I need lower power consumption on STM32CubeF0 while preserving wake-up reliability. Which low-power configuration points should be audited first (clocks, GPIO state, peripherals, wake-up sources)?</t>
@@ -1656,120 +1291,6 @@
 - middleware/BSP dependency mismatch
 ---
 If you want, I can also give you a **one-page STM32CubeF1 migration checklist template** you can reuse for every package upgrade, or a **debug flow specifically for UART/I2C/SPI/TIM/ADC**.</t>
-  </si>
-  <si>
-    <t>On STM32CubeF1, I2C sometimes gets stuck BUSY after a communication error and the bus never recovers. What is a safe software recovery sequence without full MCU reset?</t>
-  </si>
-  <si>
-    <t>Yes — on **STM32CubeF1 / STM32F1 I2C**, a common recovery for a **stuck BUSY** state after an error is to **re-initialize the I2C peripheral and, if needed, manually toggle SCL/SDA as GPIO** to release a wedged slave, **without resetting the whole MCU**.
-## Safe recovery sequence
-### 1) Stop using the peripheral
-- Disable I2C interrupts/DMA if enabled.
-- Abort any ongoing transfer in your application state machine.
-### 2) Disable the I2C peripheral
-Clear the peripheral enable bit:
-```c
-__HAL_I2C_DISABLE(&amp;hi2c1);
-```
-Or directly clear `PE` in `I2C_CR1`.
-### 3) Clear pending error flags / reset internal state
-If your software model tracks the bus state, mark it idle again and clear HAL state if appropriate.
-Typical HAL-side recovery is to set:
-- `hi2c-&gt;State = HAL_I2C_STATE_READY`
-- `hi2c-&gt;ErrorCode = HAL_I2C_ERROR_NONE`
-Be careful to do this only after the peripheral is safely disabled.
-### 4) Reconfigure the I2C pins as GPIO open-drain
-Temporarily switch:
-- `SCL` and `SDA` to **GPIO output open-drain**
-- with **pull-up** enabled if your board design supports it
-### 5) Generate clock pulses on SCL
-If a slave is holding SDA low, pulse **SCL** up to 9 times to let the slave finish its internal byte/ACK phase.
-Typical sequence:
-- Keep `SDA` released high
-- Toggle `SCL` low/high
-- Check if `SDA` is released after each pulse
-### 6) Generate a STOP condition manually
-With GPIO:
-- `SDA` low
-- `SCL` high
-- then release `SDA` high
-This helps free both master and slave state machines.
-### 7) Restore pins to I2C alternate function
-Reconfigure:
-- `SCL`, `SDA` back to I2C AF open-drain
-### 8) Re-enable and re-init I2C
-Reinitialize the peripheral with the same timing/configuration:
-```c
-HAL_I2C_Init(&amp;hi2c1);
-```
-If using Cube HAL, it may be safer to call:
-```c
-HAL_I2C_DeInit(&amp;hi2c1);
-HAL_I2C_Init(&amp;hi2c1);
-```
-## Recommended robust recovery function
-```c
-HAL_StatusTypeDef I2C1_Recover(I2C_HandleTypeDef *hi2c)
-{
-    GPIO_InitTypeDef GPIO_InitStruct = {0};
-    __disable_irq();
-    // 1) Disable I2C
-    __HAL_I2C_DISABLE(hi2c);
-    // 2) Force pins to GPIO open-drain
-    __HAL_RCC_GPIOB_CLK_ENABLE(); // adjust port as needed
-    GPIO_InitStruct.Pin = GPIO_PIN_6 | GPIO_PIN_7; // SCL/SDA example
-    GPIO_InitStruct.Mode = GPIO_MODE_OUTPUT_OD;
-    GPIO_InitStruct.Pull = GPIO_PULLUP;
-    GPIO_InitStruct.Speed = GPIO_SPEED_FREQ_HIGH;
-    HAL_GPIO_Init(GPIOB, &amp;GPIO_InitStruct);
-    // 3) Release SDA and clock SCL up to 9 pulses
-    HAL_GPIO_WritePin(GPIOB, GPIO_PIN_7, GPIO_PIN_SET); // SDA high
-    for (int i = 0; i &lt; 9; i++)
-    {
-        HAL_GPIO_WritePin(GPIOB, GPIO_PIN_6, GPIO_PIN_RESET);
-        HAL_Delay(1);
-        HAL_GPIO_WritePin(GPIOB, GPIO_PIN_6, GPIO_PIN_SET);
-        HAL_Delay(1);
-        if (HAL_GPIO_ReadPin(GPIOB, GPIO_PIN_7) == GPIO_PIN_SET)
-            break;
-    }
-    // 4) Manual STOP
-    HAL_GPIO_WritePin(GPIOB, GPIO_PIN_6, GPIO_PIN_SET);
-    HAL_GPIO_WritePin(GPIOB, GPIO_PIN_7, GPIO_PIN_RESET);
-    HAL_Delay(1);
-    HAL_GPIO_WritePin(GPIOB, GPIO_PIN_7, GPIO_PIN_SET);
-    HAL_Delay(1);
-    // 5) Restore I2C pins (AF open-drain)
-    // NOTE: replace with your Cube-generated GPIO init for I2C pins
-    MX_I2C1_GPIO_Init();
-    // 6) Reset HAL state
-    hi2c-&gt;ErrorCode = HAL_I2C_ERROR_NONE;
-    hi2c-&gt;State = HAL_I2C_STATE_READY;
-    // 7) Re-init peripheral
-    if (HAL_I2C_DeInit(hi2c) != HAL_OK) {
-        __enable_irq();
-        return HAL_ERROR;
-    }
-    if (HAL_I2C_Init(hi2c) != HAL_OK) {
-        __enable_irq();
-        return HAL_ERROR;
-    }
-    __enable_irq();
-    return HAL_OK;
-}
-```
-## Important notes for STM32F1
-- On **STM32F1 I2C**, a **BUSY flag can remain set** if the peripheral or bus was left in an invalid state.
-- If the bus lines are physically stuck low by a slave, **software only on the I2C peripheral is not enough** — you must **bit-bang recovery** on the GPIO pins.
-- If the error source is a **NACK / AF / BERR / ARLO**, clearing flags and restarting is usually enough; if the bus is truly wedged, use the GPIO recovery above.
-- Ensure the bus has proper pull-ups and that the SCL/SDA rise times meet spec.
-## Practical recommendation
-Use this escalation order:
-1. **Clear error and re-init I2C**
-2. If still BUSY, **GPIO clock pulse recovery**
-3. If still stuck, **power-cycle the external I2C slave**
-4. Only then consider **MCU reset**
-If you want, I can provide a **CubeHAL-ready recovery function for your exact I2C instance and pins**.</t>
   </si>
   <si>
     <t>I need lower power consumption on STM32CubeF1 while preserving wake-up reliability. Which low-power configuration points should be audited first (clocks, GPIO state, peripherals, wake-up sources)?</t>
@@ -2129,100 +1650,6 @@
 I can help you identify the likely breaking change very quickly.</t>
   </si>
   <si>
-    <t>On STM32CubeF2, I2C sometimes gets stuck BUSY after a communication error and the bus never recovers. What is a safe software recovery sequence without full MCU reset?</t>
-  </si>
-  <si>
-    <t>A safe recovery for a **stuck I2C BUSY** on **STM32CubeF2** is to **fully reset and reinitialize the I2C peripheral**, and, if needed, **manually free the bus lines** first. This avoids a full MCU reset in most cases.
-## Recommended recovery sequence
-### 1) Stop any ongoing I2C transfer
-Make sure your application is no longer using the peripheral:
-- abort the transfer if you are using an IRQ/DMA-based API
-- disable I2C interrupts and DMA requests
-- clear application state so no new I2C access starts during recovery
-### 2) Disable the I2C peripheral
-Clear `PE` in `I2C_CR1`:
-```c
-__HAL_I2C_DISABLE(hi2c);
-```
-### 3) Reset the I2C peripheral
-Use the peripheral reset from RCC:
-```c
-__HAL_RCC_I2C1_FORCE_RESET();
-__HAL_RCC_I2C1_RELEASE_RESET();
-```
-Use the matching instance macro for your I2C peripheral.
-### 4) Reconfigure the GPIOs if needed
-If the bus is still physically held, temporarily switch SCL/SDA to GPIO open-drain and try to release the bus by toggling SCL.
-Typical sequence:
-- set SCL and SDA as GPIO open-drain with pull-up
-- if SDA is low, generate up to **9 clock pulses** on SCL
-- then generate a **STOP** condition:
-  - drive SDA low
-  - release SCL high
-  - release SDA high
-If you have a slave stuck mid-byte or waiting for a clock edge, this often clears it.
-### 5) Reinitialize the I2C peripheral
-Call your normal init again:
-```c
-HAL_I2C_Init(&amp;hi2c);
-```
-### 6) Clear error state in software
-Reset your handle/state bookkeeping:
-- clear error codes
-- mark bus idle
-- restart any higher-level transaction queue
----
-## Safe recovery helper pattern
-```c
-HAL_StatusTypeDef I2C_Recover(I2C_HandleTypeDef *hi2c)
-{
-    __disable_irq();
-    /* Abort ongoing activity if used */
-    (void)HAL_I2C_Master_Abort_IT(hi2c);
-    /* Disable peripheral */
-    __HAL_I2C_DISABLE(hi2c);
-    /* Reset peripheral */
-    if (hi2c-&gt;Instance == I2C1)
-    {
-        __HAL_RCC_I2C1_FORCE_RESET();
-        __HAL_RCC_I2C1_RELEASE_RESET();
-    }
-#if defined(I2C2)
-    else if (hi2c-&gt;Instance == I2C2)
-    {
-        __HAL_RCC_I2C2_FORCE_RESET();
-        __HAL_RCC_I2C2_RELEASE_RESET();
-    }
-#endif
-    /* Re-init peripheral */
-    if (HAL_I2C_Init(hi2c) != HAL_OK)
-    {
-        __enable_irq();
-        return HAL_ERROR;
-    }
-    __enable_irq();
-    return HAL_OK;
-}
-```
----
-## If BUSY remains set after reset
-That usually means **the bus lines are still externally held low**, not just the peripheral state machine:
-- check SDA and SCL levels with GPIO readback
-- ensure pull-ups are present and strong enough
-- verify the slave device is powered and not in reset
-- try the **9-clock recovery** before reinitialization
----
-## Practical recommendation
-For STM32F2, the most robust approach is:
-1. **Abort transfer**
-2. **Disable I2C**
-3. **Reset I2C peripheral**
-4. **If lines are low, bit-bang 9 SCL pulses + STOP**
-5. **Reinitialize I2C**
-6. **Retry transaction**
-If you want, I can provide a **complete STM32CubeF2 recovery function** including the **GPIO bus-unwedge routine** for `I2C1` or `I2C2`.</t>
-  </si>
-  <si>
     <t>I need lower power consumption on STM32CubeF2 while preserving wake-up reliability. Which low-power configuration points should be audited first (clocks, GPIO state, peripherals, wake-up sources)?</t>
   </si>
   <si>
@@ -2590,136 +2017,6 @@
 If you want, I can turn this into a **peripheral-specific checklist** for **I2C, ADC, SPI, USART, TIM, or USB** on STM32F3.</t>
   </si>
   <si>
-    <t>On STM32CubeF3, I2C sometimes gets stuck BUSY after a communication error and the bus never recovers. What is a safe software recovery sequence without full MCU reset?</t>
-  </si>
-  <si>
-    <t>A safe recovery on **STM32CubeF3 / I2C v1 peripheral** is usually:
-1. **Abort the current transfer**
-2. **Disable the I2C peripheral**
-3. **Reconfigure the SCL/SDA pins as GPIO open-drain**
-4. **Manually clock SCL up to 9 pulses while monitoring SDA**
-5. **Generate a STOP condition in software**
-6. **Reinitialize I2C and re-enable the peripheral**
-This is the standard way to recover a stuck bus when a slave is holding **SDA low** after an error.
----
-## Recommended sequence
-### 1) Disable I2C
-Clear the peripheral and stop any ongoing transfer.
-```c
-__HAL_I2C_DISABLE(&amp;hi2c1);
-```
-If DMA/interrupts are involved, also stop them first and clear error state:
-```c
-HAL_I2C_DeInit(&amp;hi2c1);
-```
----
-### 2) Force SCL/SDA to GPIO open-drain
-Switch the two pins from I2C alternate function to GPIO open-drain with pull-up.
-- **SCL**: output open-drain
-- **SDA**: input or open-drain output
-- Keep them released high when not driven low
-This lets you manually toggle SCL even if the I2C peripheral is wedged.
----
-### 3) Clock SCL manually
-If a slave is stuck mid-byte, it may need up to **9 clock pulses** to finish shifting out its internal state.
-Pseudo-sequence:
-```c
-for (int i = 0; i &lt; 9; i++)
-{
-    // Drive SCL low
-    HAL_GPIO_WritePin(I2C_SCL_GPIO_Port, I2C_SCL_Pin, GPIO_PIN_RESET);
-    delay_us(5);
-    // Release SCL high
-    HAL_GPIO_WritePin(I2C_SCL_GPIO_Port, I2C_SCL_Pin, GPIO_PIN_SET);
-    delay_us(5);
-    // Optional: check if SDA got released
-    if (HAL_GPIO_ReadPin(I2C_SDA_GPIO_Port, I2C_SDA_Pin) == GPIO_PIN_SET)
-        break;
-}
-```
-If your bus has clock stretching, wait for SCL to actually go high before continuing.
----
-### 4) Generate a STOP condition manually
-If SDA is still low, try to create a STOP on the bus:
-- Keep SCL high
-- Transition SDA from low to high
-```c
-HAL_GPIO_WritePin(I2C_SDA_GPIO_Port, I2C_SDA_Pin, GPIO_PIN_RESET);
-delay_us(5);
-HAL_GPIO_WritePin(I2C_SCL_GPIO_Port, I2C_SCL_Pin, GPIO_PIN_SET);
-delay_us(5);
-HAL_GPIO_WritePin(I2C_SDA_GPIO_Port, I2C_SDA_Pin, GPIO_PIN_SET);
-delay_us(5);
-```
----
-### 5) Restore I2C pins and reinitialize peripheral
-Return pins to AF open-drain, then reinit the peripheral.
-```c
-HAL_I2C_Init(&amp;hi2c1);
-```
-If you used `HAL_I2C_DeInit()`, call `HAL_I2C_Init()` after GPIO is restored.
----
-## A robust recovery helper
-```c
-static void I2C_BusRecovery(I2C_HandleTypeDef *hi2c)
-{
-    GPIO_InitTypeDef GPIO_InitStruct = {0};
-    // 1. Disable peripheral
-    __HAL_I2C_DISABLE(hi2c);
-    // 2. Reconfigure pins as GPIO open-drain
-    // Enable GPIO clocks as needed here
-    GPIO_InitStruct.Pin = I2C_SCL_Pin | I2C_SDA_Pin;
-    GPIO_InitStruct.Mode = GPIO_MODE_OUTPUT_OD;
-    GPIO_InitStruct.Pull = GPIO_PULLUP;
-    GPIO_InitStruct.Speed = GPIO_SPEED_FREQ_HIGH;
-    HAL_GPIO_Init(I2C_SCL_GPIO_Port, &amp;GPIO_InitStruct);
-    HAL_GPIO_WritePin(I2C_SCL_GPIO_Port, I2C_SCL_Pin, GPIO_PIN_SET);
-    HAL_GPIO_WritePin(I2C_SDA_GPIO_Port, I2C_SDA_Pin, GPIO_PIN_SET);
-    delay_us(5);
-    // 3. Pulse SCL up to 9 times
-    for (int i = 0; i &lt; 9; i++)
-    {
-        HAL_GPIO_WritePin(I2C_SCL_GPIO_Port, I2C_SCL_Pin, GPIO_PIN_RESET);
-        delay_us(5);
-        HAL_GPIO_WritePin(I2C_SCL_GPIO_Port, I2C_SCL_Pin, GPIO_PIN_SET);
-        delay_us(5);
-        if (HAL_GPIO_ReadPin(I2C_SDA_GPIO_Port, I2C_SDA_Pin) == GPIO_PIN_SET)
-            break;
-    }
-    // 4. Generate STOP
-    HAL_GPIO_WritePin(I2C_SDA_GPIO_Port, I2C_SDA_Pin, GPIO_PIN_RESET);
-    delay_us(5);
-    HAL_GPIO_WritePin(I2C_SCL_GPIO_Port, I2C_SCL_Pin, GPIO_PIN_SET);
-    delay_us(5);
-    HAL_GPIO_WritePin(I2C_SDA_GPIO_Port, I2C_SDA_Pin, GPIO_PIN_SET);
-    delay_us(5);
-    // 5. Restore AF I2C pins elsewhere in MX_GPIO_Init() or here
-    // 6. Re-enable peripheral
-    HAL_I2C_Init(hi2c);
-}
-```
----
-## Important safety notes
-- **Do not toggle SCL while the I2C peripheral is still enabled.**
-- Make sure **both lines are pulled up** externally as required by I2C.
-- If a slave is **permanently powering down or holding SDA low due to latch-up**, software recovery may fail.
-- If the bus is shared with other masters, recovery must be coordinated.
-- If the STM32 pins are not 5V tolerant in your setup, keep recovery logic within electrical limits.
----
-## Best practice in STM32CubeF3
-In your error callback, detect bus errors like:
-- `HAL_I2C_ERROR_BERR`
-- `HAL_I2C_ERROR_ARLO`
-- `HAL_I2C_ERROR_AF`
-- `HAL_I2C_ERROR_TIMEOUT`
-Then:
-1. disable I2C
-2. perform bus recovery
-3. reinit and retry once or twice
----
-If you want, I can provide a **drop-in STM32CubeF3 recovery function** tailored to **I2C1/I2C2** with exact GPIO and clock macros.</t>
-  </si>
-  <si>
     <t>I need lower power consumption on STM32CubeF3 while preserving wake-up reliability. Which low-power configuration points should be audited first (clocks, GPIO state, peripherals, wake-up sources)?</t>
   </si>
   <si>
@@ -3030,137 +2327,6 @@
 - **DMA/IRQ mapping changed**
 ---
 If you want, I can also give you a **step-by-step STM32CubeF4 migration diff template** you can apply directly to your project files.</t>
-  </si>
-  <si>
-    <t>On STM32CubeF4, I2C sometimes gets stuck BUSY after a communication error and the bus never recovers. What is a safe software recovery sequence without full MCU reset?</t>
-  </si>
-  <si>
-    <t>A safe **software-only I2C bus recovery** on STM32CubeF4 is usually:
-## Goal
-Recover from a situation where:
-- I2C peripheral flags are stuck, especially **BUSY**
-- A transaction ended with an error
-- SDA and/or SCL may be held low by a target or by the peripheral state machine
-## Recommended recovery sequence
-### 1) Stop using the I2C peripheral
-- Disable I2C interrupts / DMA if enabled
-- Abort any ongoing transfer
-- Make sure no task is still using the bus
-### 2) Disable the I2C peripheral
-Clear the peripheral enable bit:
-```c
-__HAL_I2C_DISABLE(&amp;hi2c1);
-```
-### 3) Reconfigure SCL and SDA as GPIO open-drain
-Temporarily switch the pins to **GPIO open-drain** with **pull-up** or external pull-up support.
-Typical idea:
-- SCL = output open-drain
-- SDA = input or output open-drain
-- Both released high initially
-### 4) Manually toggle SCL to free a stuck target
-Generate up to **9 clock pulses** on SCL while watching SDA.
-Purpose:
-- If a target is mid-byte, extra clocks allow it to shift out the remaining bits and release SDA
-Procedure:
-- Drive SCL low
-- Release SCL high
-- Repeat 9 times
-- If SDA releases earlier, stop
-### 5) Generate a STOP condition manually
-After SCL is released:
-- Ensure SDA is low
-- Release SCL high
-- Then release SDA high
-This emulates an I2C STOP and often clears the target state machine.
-### 6) Restore pins to I2C alternate function
-Reconfigure SCL/SDA back to I2C AF open-drain.
-### 7) Reset and reinitialize the I2C peripheral
-Perform peripheral-level reset if needed, then re-init:
-```c
-__HAL_RCC_I2C1_FORCE_RESET();
-__HAL_RCC_I2C1_RELEASE_RESET();
-HAL_I2C_Init(&amp;hi2c1);
-```
-### 8) Clear HAL state and errors if required
-If the HAL handle remains busy/error-latched, reset its state before reusing it.
----
-# Practical recovery function
-```c
-static void I2C1_BusRecovery(void)
-{
-    GPIO_InitTypeDef GPIO_InitStruct = {0};
-    // 1. Disable I2C peripheral
-    __HAL_I2C_DISABLE(&amp;hi2c1);
-    // 2. Reconfigure SDA/SCL as GPIO open-drain
-    __HAL_RCC_GPIOB_CLK_ENABLE();
-    GPIO_InitStruct.Pin = GPIO_PIN_8 | GPIO_PIN_9;   // Example pins: PB8=SCL, PB9=SDA
-    GPIO_InitStruct.Mode = GPIO_MODE_OUTPUT_OD;
-    GPIO_InitStruct.Pull = GPIO_PULLUP;
-    GPIO_InitStruct.Speed = GPIO_SPEED_FREQ_HIGH;
-    HAL_GPIO_Init(GPIOB, &amp;GPIO_InitStruct);
-    // Release both lines high
-    HAL_GPIO_WritePin(GPIOB, GPIO_PIN_8 | GPIO_PIN_9, GPIO_PIN_SET);
-    HAL_Delay(1);
-    // 3. Clock out up to 9 pulses while SDA is held low
-    for (int i = 0; i &lt; 9; i++)
-    {
-        if (HAL_GPIO_ReadPin(GPIOB, GPIO_PIN_9) == GPIO_PIN_SET)
-            break;
-        HAL_GPIO_WritePin(GPIOB, GPIO_PIN_8, GPIO_PIN_RESET);
-        HAL_Delay(1);
-        HAL_GPIO_WritePin(GPIOB, GPIO_PIN_8, GPIO_PIN_SET);
-        HAL_Delay(1);
-    }
-    // 4. Generate STOP condition
-    HAL_GPIO_WritePin(GPIOB, GPIO_PIN_9, GPIO_PIN_RESET);
-    HAL_Delay(1);
-    HAL_GPIO_WritePin(GPIOB, GPIO_PIN_8, GPIO_PIN_SET);
-    HAL_Delay(1);
-    HAL_GPIO_WritePin(GPIOB, GPIO_PIN_9, GPIO_PIN_SET);
-    HAL_Delay(1);
-    // 5. Restore I2C AF pins
-    GPIO_InitStruct.Pin = GPIO_PIN_8 | GPIO_PIN_9;
-    GPIO_InitStruct.Mode = GPIO_MODE_AF_OD;
-    GPIO_InitStruct.Pull = GPIO_PULLUP;
-    GPIO_InitStruct.Speed = GPIO_SPEED_FREQ_VERY_HIGH;
-    GPIO_InitStruct.Alternate = GPIO_AF4_I2C1;
-    HAL_GPIO_Init(GPIOB, &amp;GPIO_InitStruct);
-    // 6. Reset I2C peripheral
-    __HAL_RCC_I2C1_FORCE_RESET();
-    __HAL_RCC_I2C1_RELEASE_RESET();
-    // 7. Reinitialize HAL
-    HAL_I2C_Init(&amp;hi2c1);
-}
-```
----
-# Important notes
-## 1) BUSY may be internal or external
-If the BUSY flag is due to:
-- a target holding SDA low
-- a malformed transfer mid-byte
-then GPIO clock pulsing helps.
-If BUSY is due to a **stuck peripheral state machine**, you may also need:
-- peripheral reset
-- reinit of HAL state
-## 2) Ensure no other master is on the bus
-If another master exists, bus recovery must coordinate with it.
-## 3) Use the actual pins and AF for your board
-The example uses **PB8/PB9** and **AF4**, which are common on STM32F4, but check your exact device/board.
-## 4) Add a timeout and fallback
-If SDA remains low after recovery:
-- the target may be truly hung
-- power-cycling that target may be required
----
-# Safer sequence summary
-1. Abort transfers and disable interrupts  
-2. Disable I2C peripheral  
-3. Reconfigure SCL/SDA as GPIO open-drain  
-4. Pulse SCL up to 9 times  
-5. Generate STOP  
-6. Reset peripheral  
-7. Reinitialize I2C  
-8. Retry transaction with timeout
-If you want, I can provide a **drop-in STM32CubeF4 bus-recovery helper** for your exact I2C instance and pin mapping.</t>
   </si>
   <si>
     <t>I need lower power consumption on STM32CubeF4 while preserving wake-up reliability. Which low-power configuration points should be audited first (clocks, GPIO state, peripherals, wake-up sources)?</t>
@@ -3570,108 +2736,6 @@
 If you want, I can also provide a **peripheral-specific migration checklist** for **UART, SPI, I2C, ADC, TIM, USB, Ethernet, or FMC** on STM32F7.</t>
   </si>
   <si>
-    <t>On STM32CubeF7, I2C sometimes gets stuck BUSY after a communication error and the bus never recovers. What is a safe software recovery sequence without full MCU reset?</t>
-  </si>
-  <si>
-    <t>A safe recovery is to **force the I2C peripheral into reset, manually free the bus lines if needed, then reinitialize**. The key is to recover both the **peripheral state** and the **physical bus state**.
-## Recommended recovery sequence
-### 1) Stop ongoing I2C activity
-- Abort any DMA/IT transfer if used.
-- Disable I2C interrupts for that instance.
-- Make sure no task is still accessing the bus.
-### 2) Disable the I2C peripheral
-```c
-__HAL_I2C_DISABLE(&amp;hi2c1);
-```
-### 3) Clear the peripheral error/state flags
-If you use HAL, clear the handle state and error code after disabling:
-```c
-hi2c1.State = HAL_I2C_STATE_READY;
-hi2c1.ErrorCode = HAL_I2C_ERROR_NONE;
-```
-### 4) Recover the bus lines manually with GPIO
-This is the important part when **SDA is held low by a slave** or the bus is left in a bad state.
-- Reconfigure **SCL and SDA as GPIO open-drain outputs**
-- Drive **SCL high/low toggles up to 9 pulses** to let a stuck slave shift out its internal state
-- Keep **SDA released high**
-- Then generate a **STOP condition**:
-  - SDA low while SCL high
-  - then SDA high while SCL high
-Typical sequence:
-```c
-// 1. Configure pins as GPIO open-drain with pull-up
-// 2. While SDA is low, toggle SCL 9 times
-// 3. Generate STOP: SDA low -&gt; SCL high -&gt; SDA high
-```
-### 5) Reconfigure pins back to I2C alternate function
-Restore the SDA/SCL pins to I2C AF mode.
-### 6) Reset and reinitialize the I2C peripheral
-Use the peripheral reset line in RCC if available:
-```c
-__HAL_RCC_I2C1_FORCE_RESET();
-__HAL_RCC_I2C1_RELEASE_RESET();
-```
-Then call:
-```c
-HAL_I2C_DeInit(&amp;hi2c1);
-HAL_I2C_Init(&amp;hi2c1);
-```
-### 7) Verify bus is free before restarting transactions
-Check both lines read high:
-- SCL = 1
-- SDA = 1
-If not, repeat the GPIO recovery.
----
-## Practical safe recovery function outline
-```c
-HAL_StatusTypeDef I2C_BusRecover(I2C_HandleTypeDef *hi2c)
-{
-    // 1. Abort activity if needed
-    HAL_I2C_DeInit(hi2c);
-    // 2. Disable peripheral
-    __HAL_I2C_DISABLE(hi2c);
-    // 3. Configure SCL/SDA as GPIO OD outputs
-    //    (application-specific pin remap/code here)
-    // 4. Clock SCL up to 9 times while SDA released
-    for (int i = 0; i &lt; 9; i++)
-    {
-        HAL_GPIO_WritePin(I2C_SCL_GPIO_Port, I2C_SCL_Pin, GPIO_PIN_RESET);
-        HAL_Delay(1);
-        HAL_GPIO_WritePin(I2C_SCL_GPIO_Port, I2C_SCL_Pin, GPIO_PIN_SET);
-        HAL_Delay(1);
-        if (HAL_GPIO_ReadPin(I2C_SDA_GPIO_Port, I2C_SDA_Pin) == GPIO_PIN_SET)
-            break;
-    }
-    // 5. Generate STOP
-    HAL_GPIO_WritePin(I2C_SDA_GPIO_Port, I2C_SDA_Pin, GPIO_PIN_RESET);
-    HAL_Delay(1);
-    HAL_GPIO_WritePin(I2C_SCL_GPIO_Port, I2C_SCL_Pin, GPIO_PIN_SET);
-    HAL_Delay(1);
-    HAL_GPIO_WritePin(I2C_SDA_GPIO_Port, I2C_SDA_Pin, GPIO_PIN_SET);
-    HAL_Delay(1);
-    // 6. Restore AF mode for I2C pins
-    //    (application-specific pin init code here)
-    // 7. Reset peripheral and reinit
-    __HAL_RCC_I2C1_FORCE_RESET();
-    __HAL_RCC_I2C1_RELEASE_RESET();
-    if (HAL_I2C_Init(hi2c) != HAL_OK)
-        return HAL_ERROR;
-    return HAL_OK;
-}
-```
----
-## Notes specific to STM32CubeF7
-- On STM32F7, the I2C peripheral is sensitive to **stuck BUSY** after missing STOP, arbitration issues, or slave clock stretching faults.
-- If the peripheral is locked in BUSY but both lines are actually high, a **peripheral reset + reinit** is usually enough.
-- If **SDA is low**, you almost always need the **manual clock-out GPIO recovery** first.
-## Best practice
-Before every transaction, you can also:
-- time out on BUSY,
-- detect line state with GPIO input,
-- run bus recovery automatically if BUSY persists too long.
-If you want, I can provide a **ready-to-use STM32CubeF7 recovery function** for a specific I2C instance, including GPIO reconfiguration code.</t>
-  </si>
-  <si>
     <t>I need lower power consumption on STM32CubeF7 while preserving wake-up reliability. Which low-power configuration points should be audited first (clocks, GPIO state, peripherals, wake-up sources)?</t>
   </si>
   <si>
@@ -4035,151 +3099,6 @@
 If you want, I can give you a **concrete STM32CubeG0 migration checklist template** or a **diff checklist for one specific peripheral** like `I2C`, `UART`, `SPI`, or `ADC`.</t>
   </si>
   <si>
-    <t>On STM32CubeG0, I2C sometimes gets stuck BUSY after a communication error and the bus never recovers. What is a safe software recovery sequence without full MCU reset?</t>
-  </si>
-  <si>
-    <t>A safe recovery pattern on **STM32CubeG0 / STM32G0 I2C** is to:
-1. **Abort the ongoing transaction**
-2. **Disable the I2C peripheral**
-3. **Manually release SCL/SDA if the bus is physically held low**
-4. **Generate bus-clear clock pulses on SCL**
-5. **Force a STOP condition if possible**
-6. **Reinitialize the I2C peripheral**
-7. **Re-enable interrupts / start normal operation**
-This is the usual approach when the peripheral remains stuck in **BUSY** after an error such as a NACK, arbitration loss, or a slave holding SDA low.
----
-## Recommended recovery sequence
-### 1) Abort the transfer
-If you use HAL, first stop any ongoing master/slave operation:
-```c
-HAL_I2C_Master_Abort_IT(&amp;hi2c1, DevAddress);
-```
-If you are in polling/blocking mode, ensure the application no longer waits on the transaction.
----
-### 2) Disable the I2C peripheral
-Clear the peripheral enable bit so the hardware FSM is reset:
-```c
-__HAL_I2C_DISABLE(&amp;hi2c1);
-```
-If needed, also clear error flags in `I2C-&gt;ICR` depending on the failure condition.
----
-### 3) Switch SCL/SDA to GPIO open-drain
-Temporarily detach the pins from I2C and drive them as GPIO open-drain with pull-up enabled externally or internally.
-- **SCL**: output open-drain
-- **SDA**: input open-drain or output open-drain depending on the strategy
-- Do **not** drive lines high actively
----
-### 4) Bus clear: toggle SCL up to 9 times
-If a slave is holding SDA low because it was mid-byte, clock the bus until it releases SDA.
-Typical sequence:
-- Set SCL low
-- Set SCL high
-- Read SDA
-- Repeat up to **9 pulses**
-If SDA is released before 9 pulses, stop pulsing.
-Conceptually:
-```c
-for (int i = 0; i &lt; 9; i++)
-{
-    SCL_LOW();
-    delay_us(5);
-    SCL_RELEASE();
-    delay_us(5);
-    if (SDA_READ() == 1)
-        break;
-}
-```
----
-### 5) Generate a STOP condition manually
-If SDA is now high, create a STOP-like transition:
-- SDA low while SCL high
-- then SDA high while SCL high
-This helps return the bus to idle.
----
-### 6) Restore I2C pin alternate function
-Put the pins back to I2C alternate function open-drain mode.
----
-### 7) Reinitialize the peripheral
-Call the normal init routine again:
-```c
-HAL_I2C_DeInit(&amp;hi2c1);
-HAL_I2C_Init(&amp;hi2c1);
-```
-If timing or filters were configured, ensure they are restored exactly as before.
----
-## Practical HAL recovery function
-```c
-HAL_StatusTypeDef I2C_Recover(I2C_HandleTypeDef *hi2c)
-{
-    GPIO_InitTypeDef GPIO_InitStruct = {0};
-    // 1. Abort and disable I2C
-    __HAL_I2C_DISABLE(hi2c);
-    // Optional: force reset of the peripheral
-    __HAL_RCC_I2C1_FORCE_RESET();
-    __HAL_RCC_I2C1_RELEASE_RESET();
-    // 2. Configure SCL/SDA as GPIO open-drain
-    // Example only: replace with your actual port/pins
-    GPIO_InitStruct.Pin = SCL_PIN | SDA_PIN;
-    GPIO_InitStruct.Mode = GPIO_MODE_OUTPUT_OD;
-    GPIO_InitStruct.Pull = GPIO_PULLUP;
-    GPIO_InitStruct.Speed = GPIO_SPEED_FREQ_HIGH;
-    HAL_GPIO_Init(SCL_SDA_GPIO_PORT, &amp;GPIO_InitStruct);
-    // 3. Bus clear pulses on SCL
-    HAL_GPIO_WritePin(SCL_GPIO_PORT, SCL_PIN, GPIO_PIN_SET);
-    HAL_GPIO_WritePin(SDA_GPIO_PORT, SDA_PIN, GPIO_PIN_SET);
-    for (int i = 0; i &lt; 9; i++)
-    {
-        HAL_GPIO_WritePin(SCL_GPIO_PORT, SCL_PIN, GPIO_PIN_RESET);
-        delay_us(5);
-        HAL_GPIO_WritePin(SCL_GPIO_PORT, SCL_PIN, GPIO_PIN_SET);
-        delay_us(5);
-        if (HAL_GPIO_ReadPin(SDA_GPIO_PORT, SDA_PIN) == GPIO_PIN_SET)
-            break;
-    }
-    // 4. Generate STOP
-    HAL_GPIO_WritePin(SDA_GPIO_PORT, SDA_PIN, GPIO_PIN_RESET);
-    delay_us(5);
-    HAL_GPIO_WritePin(SCL_GPIO_PORT, SCL_PIN, GPIO_PIN_SET);
-    delay_us(5);
-    HAL_GPIO_WritePin(SDA_GPIO_PORT, SDA_PIN, GPIO_PIN_SET);
-    delay_us(5);
-    // 5. Restore AF mode
-    GPIO_InitStruct.Pin = SCL_PIN | SDA_PIN;
-    GPIO_InitStruct.Mode = GPIO_MODE_AF_OD;
-    GPIO_InitStruct.Pull = GPIO_PULLUP;
-    GPIO_InitStruct.Speed = GPIO_SPEED_FREQ_HIGH;
-    GPIO_InitStruct.Alternate = GPIO_AF6_I2C1; // example
-    HAL_GPIO_Init(SCL_SDA_GPIO_PORT, &amp;GPIO_InitStruct);
-    // 6. Reinitialize I2C
-    if (HAL_I2C_DeInit(hi2c) != HAL_OK)
-        return HAL_ERROR;
-    if (HAL_I2C_Init(hi2c) != HAL_OK)
-        return HAL_ERROR;
-    return HAL_OK;
-}
-```
----
-## Important notes
-- If **SCL is physically low**, software recovery cannot succeed until the external device releases it.
-- If **SDA is permanently low**, the slave may be wedged or powered incorrectly.
-- Ensure pull-ups are present and the bus capacitance is within spec.
-- For robust systems, implement a **timeout + bus recovery state machine** after any I2C error.
-- Avoid repeated `HAL_I2C_Init()` calls without first disabling/resetting the peripheral, because the BUSY flag may persist in hardware state.
----
-## Best practice for STM32G0
-On STM32G0, after a bad error state, it is often safer to:
-- **disable the I2C**
-- **toggle peripheral reset in RCC**
-- **recover the bus with GPIO**
-- **re-init I2C**
-This combination is usually more reliable than only calling `HAL_I2C_DeInit()`.
----
-If you want, I can provide:
-- a **CubeMX-friendly recovery function** for `I2C1` on STM32G0,
-- an **interrupt-safe version**, or
-- a version tailored to **your exact SCL/SDA pins**.</t>
-  </si>
-  <si>
     <t>I need lower power consumption on STM32CubeG0 while preserving wake-up reliability. Which low-power configuration points should be audited first (clocks, GPIO state, peripherals, wake-up sources)?</t>
   </si>
   <si>
@@ -5078,132 +3997,6 @@
 If you want, I can also give you a **practical step-by-step STM32CubeH5 migration checklist table** or a **debug template for `HAL_ERROR` / `HAL_TIMEOUT` tracing**.</t>
   </si>
   <si>
-    <t>On STM32CubeH5, I2C sometimes gets stuck BUSY after a communication error and the bus never recovers. What is a safe software recovery sequence without full MCU reset?</t>
-  </si>
-  <si>
-    <t>A safe **software-only I2C bus recovery** on STM32CubeH5 is usually a two-part process:
-1. **Recover a possibly stuck slave/bus lines**
-2. **Reset/reinitialize the STM32 I2C peripheral cleanly**
-This avoids a full MCU reset and is typically safe if the bus is electrically healthy.
----
-## Recommended recovery sequence
-### 1) Abort any ongoing transfer
-If a HAL transfer is active or errored:
-- call `HAL_I2C_Master_Abort_IT()` / `HAL_I2C_Slave_Abort_IT()` if applicable, or
-- stop the peripheral activity and wait for the state to become `READY`
-Then:
-- disable I2C interrupts if you manage them manually
-- clear pending error flags through HAL handling or by resetting the peripheral state
----
-### 2) Disable the I2C peripheral
-Turn off the peripheral before touching GPIOs:
-```c
-__HAL_I2C_DISABLE(&amp;hi2c1);
-```
-This prevents the peripheral from fighting the bus pins.
----
-### 3) Reconfigure SCL and SDA as GPIO open-drain
-Temporarily drive the pins as GPIO open-drain with pull-ups enabled.
-- **SCL**: output open-drain
-- **SDA**: input or open-drain output depending on your recovery method
-- let the lines idle high first
-If SDA is stuck low, you need to clock SCL manually.
----
-### 4) Generate up to 9 clock pulses on SCL
-If a slave is holding SDA low, pulse SCL **9 times maximum** while monitoring SDA.
-Typical idea:
-- set SCL low
-- delay
-- set SCL high
-- delay
-- repeat up to 9 times
-Stop early if SDA releases high.
-This forces most I2C slaves to finish an interrupted byte and release the bus.
----
-### 5) Generate a STOP condition manually
-Once SDA is released:
-- ensure SCL is high
-- drive SDA low
-- then release SDA high while SCL is high
-That creates a STOP condition and leaves the bus in idle.
----
-### 6) Restore I2C pin alternate function
-Reconfigure SCL/SDA back to I2C AF mode.
----
-### 7) Reset and reinitialize the I2C peripheral
-Use peripheral reset or deinit/init sequence:
-```c
-HAL_I2C_DeInit(&amp;hi2c1);
-HAL_I2C_Init(&amp;hi2c1);
-```
-If needed, also reset the kernel clock or peripheral reset bit for a more forceful reset.
----
-## Practical recovery function example
-```c
-static void I2C_BusRecover(I2C_HandleTypeDef *hi2c)
-{
-    GPIO_InitTypeDef GPIO_InitStruct = {0};
-    // 1) Disable I2C peripheral
-    __HAL_I2C_DISABLE(hi2c);
-    // 2) Configure SCL/SDA as GPIO open-drain
-    // (replace with your actual port/pin)
-    GPIO_InitStruct.Pin = I2C1_SCL_Pin | I2C1_SDA_Pin;
-    GPIO_InitStruct.Mode = GPIO_MODE_OUTPUT_OD;
-    GPIO_InitStruct.Pull = GPIO_PULLUP;
-    GPIO_InitStruct.Speed = GPIO_SPEED_FREQ_HIGH;
-    HAL_GPIO_Init(I2C1_SCL_GPIO_Port, &amp;GPIO_InitStruct);
-    // Release both lines high
-    HAL_GPIO_WritePin(I2C1_SCL_GPIO_Port, I2C1_SCL_Pin | I2C1_SDA_Pin, GPIO_PIN_SET);
-    HAL_Delay(1);
-    // 3) Clock out stuck slave, max 9 pulses
-    for (int i = 0; i &lt; 9; i++)
-    {
-        if (HAL_GPIO_ReadPin(I2C1_SDA_GPIO_Port, I2C1_SDA_Pin) == GPIO_PIN_SET)
-            break;
-        HAL_GPIO_WritePin(I2C1_SCL_GPIO_Port, I2C1_SCL_Pin, GPIO_PIN_RESET);
-        HAL_Delay(1);
-        HAL_GPIO_WritePin(I2C1_SCL_GPIO_Port, I2C1_SCL_Pin, GPIO_PIN_SET);
-        HAL_Delay(1);
-    }
-    // 4) Generate STOP
-    HAL_GPIO_WritePin(I2C1_SCL_GPIO_Port, I2C1_SCL_Pin, GPIO_PIN_SET);
-    HAL_GPIO_WritePin(I2C1_SDA_GPIO_Port, I2C1_SDA_Pin, GPIO_PIN_RESET);
-    HAL_Delay(1);
-    HAL_GPIO_WritePin(I2C1_SDA_GPIO_Port, I2C1_SDA_Pin, GPIO_PIN_SET);
-    HAL_Delay(1);
-    // 5) Restore alternate function
-    // reconfigure pins to I2C AF in your MX_GPIO_Init or locally
-    // 6) Reinitialize I2C
-    HAL_I2C_DeInit(hi2c);
-    HAL_I2C_Init(hi2c);
-}
-```
----
-## Important notes for STM32CubeH5
-- If the BUSY flag remains set because of **internal I2C peripheral state** rather than the external bus, a **peripheral reset** is often necessary.
-- On H5, a clean sequence is usually:
-  - `HAL_I2C_DeInit()`
-  - peripheral reset via RCC reset bit if needed
-  - `HAL_I2C_Init()`
-- If the bus lines are physically stuck low by a slave due to power sequencing or brownout, software recovery may fail until that slave is also reset/powered.
----
-## Best practice in the error handler
-After a timeout or bus error:
-1. abort transfer
-2. attempt bus unstick with GPIO clock pulses
-3. generate STOP
-4. deinit/reinit I2C peripheral
-5. retry the transaction once
-6. if still failing, flag the external device/bus as faulted
----
-## Safe constraints
-- Do **not** re-enable I2C before the lines are released high.
-- Do **not** clock indefinitely; use a bounded number of pulses.
-- If multiple masters exist, coordinate recovery carefully.
-- If the slave needs a full reset pin or power-cycle, bus recovery alone may not be enough.
-If you want, I can provide a **STM32CubeH5-specific recovery function** with the exact **RCC reset register / HAL API** for `I2C1`, `I2C2`, or `I2C3`.</t>
-  </si>
-  <si>
     <t>I need lower power consumption on STM32CubeH5 while preserving wake-up reliability. Which low-power configuration points should be audited first (clocks, GPIO state, peripherals, wake-up sources)?</t>
   </si>
   <si>
@@ -5646,118 +4439,6 @@
 6. **Read release notes for the peripheral**
 ---
 If you want, I can also give you a **one-page STM32CubeH7RS migration checklist template** you can reuse per project, or a **debug tree specifically for a failing peripheral** such as **SPI, I2C, USART, ADC, USB, or SDMMC**.</t>
-  </si>
-  <si>
-    <t>On STM32CubeH7RS, I2C sometimes gets stuck BUSY after a communication error and the bus never recovers. What is a safe software recovery sequence without full MCU reset?</t>
-  </si>
-  <si>
-    <t>Below is a **safe software recovery sequence** for a stuck **I2C BUSY** condition on **STM32CubeH7RS** after a communication error, **without resetting the full MCU**.
-## Recommended recovery sequence
-### 1) Stop I2C activity first
-- Abort any ongoing transfer.
-- Disable I2C interrupts and DMA linked to the I2C instance.
-- Clear any pending I2C error/status flags if your driver layer requires it.
-In HAL terms, you typically want to ensure the peripheral is not actively driving the bus anymore before manipulating GPIO.
----
-### 2) Disable the I2C peripheral
-- Clear the I2C enable bit so the peripheral releases control of SDA/SCL.
-- Wait briefly for the disable to take effect.
-If the peripheral remains enabled, pin reconfiguration may not fully release the bus.
----
-### 3) Reconfigure SCL and SDA as GPIO open-drain
-Temporarily switch:
-- **SCL** to **GPIO output open-drain**
-- **SDA** to **GPIO open-drain**
-- Both with **pull-up** enabled if available externally or internally
-This lets software manually generate bus pulses.
----
-### 4) Clock out up to 9 pulses on SCL
-If a slave is holding SDA low because of an incomplete byte transfer, generate clock pulses on SCL to let it finish its internal state machine.
-Procedure:
-- Drive SCL low/high manually
-- Sample SDA after each pulse
-- Stop early if SDA is released
-Usually:
-- **9 pulses** is the standard maximum for 8 data bits plus ACK/NACK recovery.
----
-### 5) Generate a STOP condition manually
-If SDA is released:
-- Ensure **SCL is high**
-- Pull **SDA low**
-- Then release **SDA high** while SCL remains high
-This creates a valid STOP and resets most slave state machines.
----
-### 6) Restore I2C alternate function mode
-- Reconfigure SCL/SDA back to the I2C AF pins
-- Reinitialize the I2C peripheral
-- Re-enable interrupts/DMA if used
----
-### 7) Verify bus free state
-Before restarting traffic:
-- Check that **SCL = high**
-- Check that **SDA = high**
-- Confirm the I2C peripheral no longer reports BUSY
-If BUSY persists even after manual clocking and STOP generation, the problem may be:
-- a slave permanently holding SDA low,
-- external hardware fault,
-- or the bus requires power-cycling of the slave device.
----
-## Practical HAL-oriented recovery flow
-A common robust sequence is:
-1. `HAL_I2C_DeInit(&amp;hi2c);`
-2. Reconfigure SCL/SDA as GPIO open-drain outputs
-3. Toggle SCL up to 9 times while checking SDA
-4. Manually generate STOP
-5. Restore AF mode
-6. `HAL_I2C_Init(&amp;hi2c);`
-If your application uses an error callback, perform the recovery there only after ensuring the transfer is fully aborted.
----
-## Important safety notes
-- **Do not** toggle pins while the I2C peripheral is still enabled and actively controlling them.
-- Keep GPIO speed moderate; avoid harsh edges if the bus is shared.
-- Make sure no other master is using the bus during recovery.
-- If your board has I2C pull-ups on a switched rail, ensure the rail is still powered during recovery.
----
-## Minimal pseudocode
-```c
-void I2C_BusRecovery(I2C_HandleTypeDef *hi2c)
-{
-    // 1. Abort and disable peripheral
-    HAL_I2C_DeInit(hi2c);
-    // 2. Configure SCL/SDA as GPIO open-drain outputs
-    //    SDA input can be read to detect release
-    //    (Board-specific GPIO init required)
-    // 3. Clock out up to 9 pulses
-    for (int i = 0; i &lt; 9; i++)
-    {
-        SCL_LOW();
-        delay_us(5);
-        SCL_HIGH();
-        delay_us(5);
-        if (SDA_READ() == 1)
-            break;
-    }
-    // 4. Generate STOP
-    SDA_LOW();
-    delay_us(5);
-    SCL_HIGH();
-    delay_us(5);
-    SDA_HIGH();
-    delay_us(5);
-    // 5. Restore I2C AF pins and reinit
-    //    Board-specific AF GPIO init required
-    HAL_I2C_Init(hi2c);
-}
-```
----
-## If BUSY still never clears
-Try these checks:
-- Confirm the slave is not in reset or brownout
-- Check whether SDA is physically shorted low
-- Verify pull-up values and bus rise time
-- Inspect if another master or debug circuitry is holding the line
-- Power-cycle only the affected slave, if possible
-If you want, I can provide a **STM32CubeH7RS-ready recovery function** for a specific I2C instance and pin pair.</t>
   </si>
   <si>
     <t>I need lower power consumption on STM32CubeH7RS while preserving wake-up reliability. Which low-power configuration points should be audited first (clocks, GPIO state, peripherals, wake-up sources)?</t>
@@ -6083,118 +4764,6 @@
 5. **Run minimal repro**
 6. **Compare peripheral registers before/after init**
 If you want, I can give you a **peripheral-specific migration checklist** for **I2C / SPI / UART / ADC / TIM / LPTIM / RTC / DMA** on STM32L0.</t>
-  </si>
-  <si>
-    <t>On STM32CubeL0, I2C sometimes gets stuck BUSY after a communication error and the bus never recovers. What is a safe software recovery sequence without full MCU reset?</t>
-  </si>
-  <si>
-    <t>A safe **software recovery** for an STM32L0 I2C peripheral that is stuck **BUSY** after an error is to:
-1. **Disable the I2C peripheral**
-2. **Release the I2C pins to GPIO open-drain**
-3. **Manually clock the bus to free a stuck slave**
-4. **Generate a STOP condition**
-5. **Reinitialize the I2C peripheral**
-This is the standard “bus recovery” approach when the peripheral itself is no longer able to clear the condition.
----
-## Recommended recovery sequence
-### 1) Stop I2C activity and disable the peripheral
-- Abort any ongoing transfer.
-- Disable I2C:
-  - `__HAL_I2C_DISABLE(&amp;hi2c);`
-- Clear error state in your software state machine if needed.
-### 2) Reconfigure SCL and SDA as GPIO open-drain
-Temporarily **take control of the pins as GPIO**:
-- Configure both pins as:
-  - **Open-drain**
-  - **No pull-up** if external pull-ups exist, otherwise use pull-up as needed
-  - **Output high** initially
-This lets you manually drive clocks on SCL.
-### 3) Clock out up to 9 pulses on SCL
-If a slave is holding SDA low, toggle SCL **9 times max**:
-- Set SCL low
-- Set SCL high
-- Read SDA after each pulse
-- Stop early if SDA is released high
-Why 9?  
-A stuck I2C slave may be waiting for the remaining bits of a byte plus ACK; 9 clocks usually advances it to a state where it releases SDA.
-### 4) Generate a STOP condition manually
-If SDA is free:
-- Drive SDA low while SCL is high
-- Then release SDA high while SCL remains high
-This simulates a valid STOP and puts slaves back to idle.
-### 5) Reinitialize I2C
-- Restore pins to alternate function I2C
-- Re-enable I2C
-- Reconfigure the peripheral with `HAL_I2C_Init()` or your normal init path
----
-## Practical recovery pseudocode
-```c
-void I2C_BusRecovery(I2C_HandleTypeDef *hi2c)
-{
-    GPIO_InitTypeDef GPIO_InitStruct = {0};
-    // 1. Disable I2C
-    __HAL_I2C_DISABLE(hi2c);
-    // 2. Configure SCL/SDA as GPIO open-drain outputs
-    //    Example only: replace with your actual ports/pins
-    HAL_GPIO_DeInit(I2C_SCL_GPIO_Port, I2C_SCL_Pin);
-    HAL_GPIO_DeInit(I2C_SDA_GPIO_Port, I2C_SDA_Pin);
-    GPIO_InitStruct.Pin = I2C_SCL_Pin | I2C_SDA_Pin;
-    GPIO_InitStruct.Mode = GPIO_MODE_OUTPUT_OD;
-    GPIO_InitStruct.Pull = GPIO_PULLUP;   // or NOPULL if external pull-ups exist
-    GPIO_InitStruct.Speed = GPIO_SPEED_FREQ_LOW;
-    HAL_GPIO_Init(I2C_SCL_GPIO_Port, &amp;GPIO_InitStruct);
-    // Release both lines high
-    HAL_GPIO_WritePin(I2C_SCL_GPIO_Port, I2C_SCL_Pin, GPIO_PIN_SET);
-    HAL_GPIO_WritePin(I2C_SDA_GPIO_Port, I2C_SDA_Pin, GPIO_PIN_SET);
-    HAL_Delay(1);
-    // 3. Clock SCL up to 9 times if SDA is stuck low
-    for (int i = 0; i &lt; 9; i++)
-    {
-        if (HAL_GPIO_ReadPin(I2C_SDA_GPIO_Port, I2C_SDA_Pin) == GPIO_PIN_SET)
-            break;
-        HAL_GPIO_WritePin(I2C_SCL_GPIO_Port, I2C_SCL_Pin, GPIO_PIN_RESET);
-        HAL_Delay(1);
-        HAL_GPIO_WritePin(I2C_SCL_GPIO_Port, I2C_SCL_Pin, GPIO_PIN_SET);
-        HAL_Delay(1);
-    }
-    // 4. Generate STOP: SDA low -&gt; SCL high -&gt; SDA high
-    HAL_GPIO_WritePin(I2C_SDA_GPIO_Port, I2C_SDA_Pin, GPIO_PIN_RESET);
-    HAL_Delay(1);
-    HAL_GPIO_WritePin(I2C_SCL_GPIO_Port, I2C_SCL_Pin, GPIO_PIN_SET);
-    HAL_Delay(1);
-    HAL_GPIO_WritePin(I2C_SDA_GPIO_Port, I2C_SDA_Pin, GPIO_PIN_SET);
-    HAL_Delay(1);
-    // 5. Restore I2C alternate function and re-init
-    HAL_GPIO_DeInit(I2C_SCL_GPIO_Port, I2C_SCL_Pin);
-    HAL_GPIO_DeInit(I2C_SDA_GPIO_Port, I2C_SDA_Pin);
-    // Reconfigure pins to I2C AF in your MSP init or board init
-    HAL_I2C_Init(hi2c);
-}
-```
----
-## Important notes for STM32CubeL0
-- If the **BUSY flag remains set inside the peripheral** even after the external bus is freed, you may need to:
-  - Disable the peripheral
-  - Perform a peripheral reset via RCC if available for that instance
-  - Then re-init
-For STM32L0, a **peripheral reset** is still **not a full MCU reset** and is often acceptable if software recovery alone does not clear the internal state.
----
-## Recommended robust handling
-In practice, use this order:
-1. Timeout/error detected in transaction  
-2. Abort transfer  
-3. Disable I2C  
-4. Bus recovery by GPIO clock pulses + STOP  
-5. Re-enable and re-init I2C  
-6. If still BUSY, perform **I2C peripheral reset**  
-7. Retry communication
----
-## Extra precaution
-Before starting recovery, verify:
-- SCL can actually be driven high
-- SDA is not permanently shorted low by hardware
-- Pull-ups are present and sized correctly
-If you want, I can also provide a **CubeHAL-ready STM32L0 recovery function** using your specific I2C instance and pins.</t>
   </si>
   <si>
     <t>I need lower power consumption on STM32CubeL0 while preserving wake-up reliability. Which low-power configuration points should be audited first (clocks, GPIO state, peripherals, wake-up sources)?</t>
@@ -6566,159 +5135,6 @@
 - a **debug macro snippet** to log HAL init failures quickly</t>
   </si>
   <si>
-    <t>On STM32CubeL1, I2C sometimes gets stuck BUSY after a communication error and the bus never recovers. What is a safe software recovery sequence without full MCU reset?</t>
-  </si>
-  <si>
-    <t>Yes — on **STM32CubeL1 / STM32L1 I2C v1 peripheral**, a bus error can leave the peripheral or the external bus in a **BUSY** state. A **safe software recovery** is to:
-1. **Abort the ongoing transfer**
-2. **Disable the I2C peripheral**
-3. **Recover the external bus by toggling SCL manually**
-4. **Generate a STOP condition if possible**
-5. **Reinitialize and re-enable I2C**
-This avoids a full MCU reset and is the standard approach when a slave holds **SDA low** after an error.
----
-## Recommended recovery sequence
-### 1) Stop the current I2C activity
-If using interrupts/IT/DMA:
-- Abort DMA streams if used
-- Disable I2C event/error interrupts
-- Clear pending error flags
-If using HAL:
-- Call the corresponding abort/stop logic if available in your code base
-- Make sure no I2C transfer is still running
----
-### 2) Disable the I2C peripheral
-Put the peripheral in software reset / disable mode so it stops driving the bus.
-Typical action:
-- Clear the **PE** bit in `I2C_CR1`
-This is important before GPIO bus recovery.
----
-### 3) Reconfigure SCL and SDA as GPIO open-drain
-Temporarily take control of the pins as GPIO:
-- SCL: output open-drain
-- SDA: input open-drain or output open-drain depending on your recovery method
-- External pull-ups must remain present
----
-### 4) Manually clock SCL up to 9 pulses
-If a slave is stuck mid-byte, it may be waiting for clock edges. Toggle **SCL** manually:
-- Send **up to 9 pulses**
-- After each pulse, check whether **SDA has been released high**
-- If SDA becomes high early, stop pulsing
-This often frees a slave that was holding SDA low.
----
-### 5) Generate a STOP condition manually
-Once SDA is high:
-- Drive SDA low while SCL is high
-- Then release SDA high while SCL is high
-This creates a valid **STOP** on the bus.
----
-### 6) Restore I2C pins and peripheral
-- Reconfigure pins back to I2C alternate function open-drain
-- Re-enable the I2C peripheral
-- Reinitialize HAL I2C state if used
-- Clear status/state variables in your driver
----
-## Practical recovery flow
-```text
-Error detected
-   ↓
-Abort ongoing transfer / disable IRQs
-   ↓
-Disable I2C peripheral
-   ↓
-Switch SCL/SDA to GPIO open-drain
-   ↓
-Pulse SCL up to 9 times while monitoring SDA
-   ↓
-If SDA released, generate STOP
-   ↓
-Restore AF I2C pins
-   ↓
-Re-enable and reinit I2C
-```
----
-## Important details for STM32L1
-### If BUSY remains set internally
-On older STM32 I2C IP, the **BUSY flag** may remain set if:
-- SDA was low during peripheral enable
-- A previous transfer ended abnormally
-- The bus was not properly released by a slave
-In that case, **toggling SCL/SDA externally** is usually the only reliable recovery without resetting the MCU.
-### If SDA is physically held low
-If after 9 pulses SDA is still low, the slave may be:
-- Powered down incorrectly
-- In a fault state
-- Needing a device-specific reset sequence
-Then software-only recovery may not be possible, but you can still:
-- power-cycle the slave
-- toggle the slave reset pin if available
-- reattempt bus recovery after slave reset
----
-## Example recovery code outline
-```c
-void I2C_BusRecover(I2C_TypeDef *I2Cx)
-{
-    GPIO_InitTypeDef GPIO_InitStruct = {0};
-    // 1. Disable I2C peripheral
-    I2Cx-&gt;CR1 &amp;= ~I2C_CR1_PE;
-    // 2. Configure SCL/SDA as GPIO open-drain
-    //    (replace GPIOx/pins with your board-specific mapping)
-    // GPIO_InitStruct.Pin = SCL_PIN | SDA_PIN;
-    // GPIO_InitStruct.Mode = GPIO_MODE_OUTPUT_OD;
-    // GPIO_InitStruct.Pull = GPIO_PULLUP;
-    // HAL_GPIO_Init(GPIOx, &amp;GPIO_InitStruct);
-    // 3. Release both lines high
-    // HAL_GPIO_WritePin(GPIOx, SCL_PIN | SDA_PIN, GPIO_PIN_SET);
-    // 4. Pulse SCL up to 9 times
-    for (int i = 0; i &lt; 9; i++)
-    {
-        // Drive SCL low
-        // HAL_GPIO_WritePin(GPIOx, SCL_PIN, GPIO_PIN_RESET);
-        delay_us(5);
-        // Release SCL high
-        // HAL_GPIO_WritePin(GPIOx, SCL_PIN, GPIO_PIN_SET);
-        delay_us(5);
-        // If SDA is high, bus may be free
-        // if (HAL_GPIO_ReadPin(GPIOx, SDA_PIN) == GPIO_PIN_SET)
-        //     break;
-    }
-    // 5. Generate STOP if SDA released
-    // if (HAL_GPIO_ReadPin(GPIOx, SDA_PIN) == GPIO_PIN_SET)
-    // {
-    //     HAL_GPIO_WritePin(GPIOx, SDA_PIN, GPIO_PIN_RESET);
-    //     delay_us(5);
-    //     HAL_GPIO_WritePin(GPIOx, SCL_PIN, GPIO_PIN_SET);
-    //     delay_us(5);
-    //     HAL_GPIO_WritePin(GPIOx, SDA_PIN, GPIO_PIN_SET);
-    //     delay_us(5);
-    // }
-    // 6. Restore I2C pins AF open-drain
-    // HAL_GPIO_DeInit(GPIOx, SCL_PIN | SDA_PIN);
-    // ... configure AF I2C ...
-    // 7. Re-enable I2C peripheral
-    I2Cx-&gt;CR1 |= I2C_CR1_PE;
-}
-```
----
-## Best practices
-- Call recovery **only after a real bus fault**
-- Ensure **interrupts/DMA are stopped** before switching pins to GPIO
-- Keep **timeouts** in all I2C transactions
-- Use **delays in the microsecond range** for manual clocking
-- If your board allows it, add a **slave reset GPIO** or **power switch** for unrecoverable devices
----
-## HAL note
-If you are using STM32Cube HAL, it’s often best to combine:
-- `HAL_I2C_DeInit()`
-- GPIO bus recovery
-- `HAL_I2C_Init()`
-but **deinit alone is usually not sufficient** if the external bus is still stuck.
----
-If you want, I can provide:
-1. a **ready-to-use STM32L1 HAL recovery function**, or  
-2. a version tailored to **a specific STM32L1 board/pinout**.</t>
-  </si>
-  <si>
     <t>I need lower power consumption on STM32CubeL1 while preserving wake-up reliability. Which low-power configuration points should be audited first (clocks, GPIO state, peripherals, wake-up sources)?</t>
   </si>
   <si>
@@ -7167,143 +5583,6 @@
 If you want, I can also provide a **peripheral-specific migration checklist** for **UART / I2C / SPI / ADC / TIM / DMA / USB / RTC**, or a **debug template** you can paste into your project to log the exact failing step.</t>
   </si>
   <si>
-    <t>On STM32CubeL4, I2C sometimes gets stuck BUSY after a communication error and the bus never recovers. What is a safe software recovery sequence without full MCU reset?</t>
-  </si>
-  <si>
-    <t>A safe software recovery for a **stuck I2C BUSY** on STM32CubeL4 is to:
-1. **Disable the I2C peripheral**
-2. **Recover the bus at GPIO level** by toggling **SCL** up to 9 times while checking **SDA**
-3. **Generate a STOP condition** if possible
-4. **Re-enable I2C**
-5. **Clear/restore HAL state and error flags**
-6. **Retry the transaction**
-This is the standard approach when a slave holds SDA low after an aborted transfer.
----
-## Recommended recovery sequence
-### 1) Abort any ongoing transfer
-If you use HAL in interrupt/DMA mode, first stop activity:
-- `HAL_I2C_Master_Abort_IT()` if applicable
-- Disable I2C IRQs / DMA channels
-- Make sure no task is still using the handle
----
-### 2) Disable the I2C peripheral
-Clear `PE` so the lines can be controlled as GPIO:
-```c
-__HAL_I2C_DISABLE(&amp;hi2c1);
-```
-You may also want to clear pending flags by reading/writing registers only if needed, but **do not** rely on this alone for a BUSY lock caused by the bus lines themselves.
----
-### 3) Reconfigure SCL and SDA as GPIO open-drain
-Set both pins to **GPIO open-drain**, pulled up, and drive them high by releasing them.
-Then perform clock pulses on **SCL**:
-- Keep **SDA released high**
-- Toggle **SCL** low/high up to **9 times**
-- After each pulse, check whether **SDA** is released
-If SDA is still low after 9 pulses, the slave is likely still internally stuck or the bus is physically held low.
----
-### 4) Generate a STOP condition manually
-If SDA is observed high during recovery:
-- Drive **SDA low**
-- Release **SCL high**
-- Release **SDA high**
-This creates a STOP and should free most slaves.
----
-## Example recovery code
-```c
-static void I2C1_SoftwareBusRecovery(void)
-{
-    GPIO_InitTypeDef GPIO_InitStruct = {0};
-    // 1) Disable I2C peripheral
-    __HAL_I2C_DISABLE(&amp;hi2c1);
-    // 2) Reconfigure SCL/SDA as GPIO open-drain
-    __HAL_RCC_GPIOB_CLK_ENABLE();
-    GPIO_InitStruct.Pin = GPIO_PIN_6 | GPIO_PIN_7;   // Example: PB6=SCL, PB7=SDA
-    GPIO_InitStruct.Mode = GPIO_MODE_OUTPUT_OD;
-    GPIO_InitStruct.Pull = GPIO_PULLUP;
-    GPIO_InitStruct.Speed = GPIO_SPEED_FREQ_HIGH;
-    HAL_GPIO_Init(GPIOB, &amp;GPIO_InitStruct);
-    // Release lines high
-    HAL_GPIO_WritePin(GPIOB, GPIO_PIN_6 | GPIO_PIN_7, GPIO_PIN_SET);
-    HAL_Delay(1);
-    // 3) Clock out up to 9 pulses on SCL
-    for (int i = 0; i &lt; 9; i++)
-    {
-        if (HAL_GPIO_ReadPin(GPIOB, GPIO_PIN_7) == GPIO_PIN_SET)
-        {
-            break; // SDA released
-        }
-        HAL_GPIO_WritePin(GPIOB, GPIO_PIN_6, GPIO_PIN_RESET);
-        HAL_Delay(1);
-        HAL_GPIO_WritePin(GPIOB, GPIO_PIN_6, GPIO_PIN_SET);
-        HAL_Delay(1);
-    }
-    // 4) Generate STOP condition if SDA is high
-    if (HAL_GPIO_ReadPin(GPIOB, GPIO_PIN_7) == GPIO_PIN_SET)
-    {
-        HAL_GPIO_WritePin(GPIOB, GPIO_PIN_7, GPIO_PIN_RESET);
-        HAL_Delay(1);
-        HAL_GPIO_WritePin(GPIOB, GPIO_PIN_6, GPIO_PIN_SET);
-        HAL_Delay(1);
-        HAL_GPIO_WritePin(GPIOB, GPIO_PIN_7, GPIO_PIN_SET);
-        HAL_Delay(1);
-    }
-    // 5) Restore I2C pins to alternate function
-    GPIO_InitStruct.Pin = GPIO_PIN_6 | GPIO_PIN_7;
-    GPIO_InitStruct.Mode = GPIO_MODE_AF_OD;
-    GPIO_InitStruct.Pull = GPIO_PULLUP;
-    GPIO_InitStruct.Speed = GPIO_SPEED_FREQ_VERY_HIGH;
-    GPIO_InitStruct.Alternate = GPIO_AF4_I2C1;
-    HAL_GPIO_Init(GPIOB, &amp;GPIO_InitStruct);
-    // 6) Re-enable I2C
-    __HAL_I2C_ENABLE(&amp;hi2c1);
-    // 7) Restore HAL state if needed
-    hi2c1.ErrorCode = HAL_I2C_ERROR_NONE;
-    hi2c1.State = HAL_I2C_STATE_READY;
-}
-```
----
-## Important notes for STM32L4
-### Use the correct pin mapping
-Replace `PB6/PB7` and `GPIO_AF4_I2C1` with the actual pins/peripheral instance used by your board.
-### Don’t forget pull-ups
-I2C recovery works only if the bus has valid pull-ups. External pull-ups are strongly recommended.
-### If the bus is still busy after GPIO recovery
-Then one of these is likely true:
-- a slave is truly stuck holding **SDA low**
-- **SCL** is held low by a device
-- a hardware fault exists on the bus
-- the lines are not configured correctly as open-drain with pull-ups
-If **SCL is low**, software recovery is much harder because you cannot generate clocks.
----
-## More robust approach
-Before re-enabling the peripheral, you can also force an **I2C peripheral reset**:
-```c
-__HAL_RCC_I2C1_FORCE_RESET();
-__HAL_RCC_I2C1_RELEASE_RESET();
-```
-This does **not** replace bus recovery, but it can help clear internal peripheral state.
----
-## Practical recovery order
-A good sequence is:
-1. Stop DMA/IT transfers
-2. `__HAL_I2C_DISABLE()`
-3. GPIO bit-bang SCL up to 9 pulses
-4. Create STOP condition
-5. Reset I2C peripheral block if needed
-6. Reinitialize/enable I2C
-7. Clear HAL error/state
-8. Retry transaction
----
-## If you want the safest production pattern
-Implement recovery as a dedicated function that is called when:
-- `HAL_I2C_ERROR_BERR`
-- `HAL_I2C_ERROR_ARLO`
-- `HAL_I2C_ERROR_AF`
-- `HAL_I2C_ERROR_TIMEOUT`
-- or `HAL_I2C_GetState()` remains busy too long
-If you want, I can provide a **STM32CubeL4-ready recovery function** for a specific I2C instance and pinout, including HAL callback integration.</t>
-  </si>
-  <si>
     <t>I need lower power consumption on STM32CubeL4 while preserving wake-up reliability. Which low-power configuration points should be audited first (clocks, GPIO state, peripherals, wake-up sources)?</t>
   </si>
   <si>
@@ -7680,120 +5959,6 @@
 - User code got overwritten during regeneration
 ---
 If you want, I can also give you a **one-page STM32CubeL5 migration checklist template** you can use during regression analysis.</t>
-  </si>
-  <si>
-    <t>On STM32CubeL5, I2C sometimes gets stuck BUSY after a communication error and the bus never recovers. What is a safe software recovery sequence without full MCU reset?</t>
-  </si>
-  <si>
-    <t>A safe recovery on **STM32CubeL5 I2C** is usually:
-1. **Abort the ongoing transfer**
-2. **Disable the I2C peripheral**
-3. **Temporarily reconfigure SCL/SDA as GPIO open-drain**
-4. **Manually clock SCL to release a stuck slave**
-5. **Generate a STOP condition in GPIO mode**
-6. **Restore I2C pins and reinitialize the peripheral**
-7. **Clear and re-enable interrupts / DMA state**
-## Recommended recovery sequence
-### 1) Stop any ongoing HAL transfer
-If you use HAL, first abort the peripheral to stop internal state machines:
-```c
-HAL_I2C_Master_Abort_IT(&amp;hi2c1, DevAddress);
-```
-If that is not applicable, at least make sure no transfer is still running and disable I2C interrupts/DMA linked to it.
----
-### 2) Disable the I2C peripheral
-```c
-__HAL_I2C_DISABLE(&amp;hi2c1);
-```
-If needed, also clear the software state in your application before restarting.
----
-### 3) Reconfigure SCL/SDA as GPIO open-drain
-Set both pins as **GPIO open-drain outputs** with pull-up enabled, then release them high.
-This lets you manually drive the bus without relying on the I2C peripheral.
----
-### 4) Free a slave holding SDA low by clocking SCL
-If **SDA is stuck low**, toggle **SCL** about **9 pulses** while keeping SDA released high.
-Typical sequence:
-- SDA = high
-- Generate 9 SCL pulses
-- Check if SDA releases
-This is the standard way to recover a slave that is waiting for more clocks after an aborted byte.
----
-### 5) Generate a STOP condition manually
-While SCL is high, switch SDA from low to high:
-- SDA low
-- SCL high
-- SDA high
-This helps restore idle bus state.
----
-### 6) Restore alternate-function I2C pins
-Reconfigure SCL/SDA back to I2C AF open-drain, then restart the peripheral:
-```c
-HAL_I2C_Init(&amp;hi2c1);
-```
-If you use MSP init, you may need to call your low-level init again if the pins were changed manually.
----
-### 7) Clear error flags and restart communication
-After re-init, make sure the HAL handle is back to `READY`, and discard any pending transaction state in your application.
----
-## Practical recovery helper
-```c
-static void I2C_BusRecover(I2C_HandleTypeDef *hi2c)
-{
-    GPIO_InitTypeDef GPIO_InitStruct = {0};
-    __HAL_I2C_DISABLE(hi2c);
-    // 1) Disable interrupts/DMA if used
-    __HAL_I2C_DISABLE_IT(hi2c, I2C_IT_ERRI | I2C_IT_TCI | I2C_IT_STOPI | I2C_IT_NACKI);
-    if (hi2c-&gt;hdmarx) __HAL_DMA_DISABLE(hi2c-&gt;hdmarx);
-    if (hi2c-&gt;hdmatx) __HAL_DMA_DISABLE(hi2c-&gt;hdmatx);
-    // 2) Configure SCL/SDA as GPIO OD
-    // Replace with your port/pin definitions
-    GPIO_InitStruct.Pin = I2C1_SCL_PIN | I2C1_SDA_PIN;
-    GPIO_InitStruct.Mode = GPIO_MODE_OUTPUT_OD;
-    GPIO_InitStruct.Pull = GPIO_PULLUP;
-    GPIO_InitStruct.Speed = GPIO_SPEED_FREQ_HIGH;
-    HAL_GPIO_Init(I2C1_GPIO_PORT, &amp;GPIO_InitStruct);
-    // Release lines high
-    HAL_GPIO_WritePin(I2C1_GPIO_PORT, I2C1_SCL_PIN | I2C1_SDA_PIN, GPIO_PIN_SET);
-    HAL_Delay(1);
-    // 3) Pulse SCL up to 9 times if SDA is low
-    for (int i = 0; i &lt; 9; i++)
-    {
-        if (HAL_GPIO_ReadPin(I2C1_GPIO_PORT, I2C1_SDA_PIN) == GPIO_PIN_SET)
-            break;
-        HAL_GPIO_WritePin(I2C1_GPIO_PORT, I2C1_SCL_PIN, GPIO_PIN_RESET);
-        HAL_Delay(1);
-        HAL_GPIO_WritePin(I2C1_GPIO_PORT, I2C1_SCL_PIN, GPIO_PIN_SET);
-        HAL_Delay(1);
-    }
-    // 4) Generate STOP
-    HAL_GPIO_WritePin(I2C1_GPIO_PORT, I2C1_SDA_PIN, GPIO_PIN_RESET);
-    HAL_GPIO_WritePin(I2C1_GPIO_PORT, I2C1_SCL_PIN, GPIO_PIN_SET);
-    HAL_Delay(1);
-    HAL_GPIO_WritePin(I2C1_GPIO_PORT, I2C1_SDA_PIN, GPIO_PIN_SET);
-    HAL_Delay(1);
-    // 5) Restore I2C AF pins
-    HAL_I2C_DeInit(hi2c);
-    HAL_I2C_Init(hi2c);
-}
-```
----
-## Important notes for STM32L5
-- If the I2C peripheral is stuck due to **internal BUSY state** but the bus is actually free, a **peripheral re-init** may be enough.
-- If **SDA is physically held low**, you usually need the **GPIO clock-pulse recovery**.
-- If a slave is truly wedged, recovery may still fail unless power-cycled.
-- Make sure your pull-ups and bus timing are correct; weak pull-ups are a common cause of recovery problems.
----
-## Safe usage pattern
-I recommend this order:
-1. Detect error or timeout
-2. Abort HAL transaction
-3. Disable I2C
-4. GPIO bus recovery
-5. Re-init I2C
-6. Retry transaction once
-7. Escalate if still failing
-If you want, I can provide a **CubeL5-ready recovery function** tailored to your exact I2C instance and pin mapping.</t>
   </si>
   <si>
     <t>I need lower power consumption on STM32CubeL5 while preserving wake-up reliability. Which low-power configuration points should be audited first (clocks, GPIO state, peripherals, wake-up sources)?</t>
@@ -8176,101 +6341,6 @@
 - Enable compiler warnings as errors for migration cleanup
 ---
 If you want, I can also give you a **peripheral-specific migration checklist** for **UART / I2C / SPI / ADC / TIM / DMA / USB / ETH / FMC**, or help you analyze a **specific failing init function and error code**.</t>
-  </si>
-  <si>
-    <t>On STM32CubeN6, I2C sometimes gets stuck BUSY after a communication error and the bus never recovers. What is a safe software recovery sequence without full MCU reset?</t>
-  </si>
-  <si>
-    <t>A safe recovery is to **fully de-initialize the I2C peripheral, manually release the bus with GPIO, then re-initialize**. The exact sequence that is usually robust on STM32CubeN6 is:
-## 1) Stop I2C activity and disable interrupts/DMA
-- Abort any ongoing transfer
-- Disable I2C event/error interrupts
-- Stop DMA linked to I2C, if used
-## 2) Disable the I2C peripheral
-Put the peripheral in reset-like state through HAL:
-```c
-HAL_I2C_DeInit(&amp;hi2c1);
-```
-If the peripheral remains BUSY, do not rely on it yet.
-## 3) Reconfigure SCL/SDA as open-drain GPIOs
-Temporarily switch the pins from I2C AF to **GPIO output open-drain with pull-up**.
-## 4) Generate bus-unlock pulses on SCL
-If **SDA is stuck low**, pulse **SCL** about 9 times while monitoring SDA:
-- Drive SCL low/high manually
-- Keep SDA released/high
-- If a slave was mid-byte, these clocks usually let it complete and release SDA
-Typical rule:
-- 9 pulses minimum
-- optionally stop earlier if SDA goes high
-## 5) Generate a STOP condition manually
-With both lines released high, force a software STOP:
-- SDA low while SCL high
-- then SDA high while SCL high
-This helps reset the state machine of some slaves.
-## 6) Restore I2C alternate function
-Reconfigure pins back to I2C AF, then:
-```c
-HAL_I2C_Init(&amp;hi2c1);
-```
-## 7) Clear flags and restart communication
-After re-init, retry transaction from a clean state.
----
-## Recommended recovery helper
-A practical implementation flow:
-```c
-HAL_StatusTypeDef I2C_BusRecover(I2C_HandleTypeDef *hi2c)
-{
-    GPIO_InitTypeDef GPIO_InitStruct = {0};
-    __HAL_I2C_DISABLE(hi2c);
-    // Stop interrupts / DMA if used in your project
-    // HAL_I2C_EnableListen_IT(...) off, HAL_DMA_Abort(...), etc.
-    HAL_I2C_DeInit(hi2c);
-    // 1) Configure SCL/SDA as GPIO open-drain outputs with pull-up
-    //    (replace with your actual port/pin)
-    GPIO_InitStruct.Pin = I2C_SCL_Pin | I2C_SDA_Pin;
-    GPIO_InitStruct.Mode = GPIO_MODE_OUTPUT_OD;
-    GPIO_InitStruct.Pull = GPIO_PULLUP;
-    GPIO_InitStruct.Speed = GPIO_SPEED_FREQ_HIGH;
-    HAL_GPIO_Init(I2C_GPIO_Port, &amp;GPIO_InitStruct);
-    // Release both lines
-    HAL_GPIO_WritePin(I2C_GPIO_Port, I2C_SCL_Pin | I2C_SDA_Pin, GPIO_PIN_SET);
-    HAL_Delay(1);
-    // 2) If SDA is low, clock SCL up to 9 times
-    for (int i = 0; i &lt; 9 &amp;&amp; HAL_GPIO_ReadPin(I2C_GPIO_Port, I2C_SDA_Pin) == GPIO_PIN_RESET; i++)
-    {
-        HAL_GPIO_WritePin(I2C_GPIO_Port, I2C_SCL_Pin, GPIO_PIN_RESET);
-        delay_us(5);
-        HAL_GPIO_WritePin(I2C_GPIO_Port, I2C_SCL_Pin, GPIO_PIN_SET);
-        delay_us(5);
-    }
-    // 3) Generate STOP: SDA low while SCL high, then SDA high
-    HAL_GPIO_WritePin(I2C_GPIO_Port, I2C_SDA_Pin, GPIO_PIN_RESET);
-    delay_us(5);
-    HAL_GPIO_WritePin(I2C_GPIO_Port, I2C_SCL_Pin, GPIO_PIN_SET);
-    delay_us(5);
-    HAL_GPIO_WritePin(I2C_GPIO_Port, I2C_SDA_Pin, GPIO_PIN_SET);
-    delay_us(5);
-    // 4) Restore AF I2C pins
-    //    Reconfigure through MX_GPIO_Init() or explicit AF init
-    MX_I2C1_Init();   // or HAL_I2C_Init(hi2c)
-    return HAL_OK;
-}
-```
----
-## Important notes for STM32CubeN6
-- If you use **I2C in interrupt/DMA mode**, additional cleanup may be needed before re-init:
-  - abort DMA streams/channels
-  - clear error state in your driver logic
-  - reset application state machine
-- Make sure the GPIOs really become **open-drain** during recovery; driving push-pull can damage the bus.
-- If an external device holds **SCL low** due to clock stretching or a fault, software recovery may not work. In that case the slave may need its own reset or power cycle.
-- Keep the recovery routine in a **timeout-protected path** so it never blocks indefinitely.
-## Best practice
-Use this sequence after:
-- `HAL_I2C_ErrorCallback()`
-- `HAL_TIMEOUT`
-- detection of `HAL_I2C_STATE_BUSY` lingering longer than expected
-If you want, I can provide a **CubeN6-ready recovery function** tailored to your exact I2C instance and pins.</t>
   </si>
   <si>
     <t>I need lower power consumption on STM32CubeN6 while preserving wake-up reliability. Which low-power configuration points should be audited first (clocks, GPIO state, peripherals, wake-up sources)?</t>
@@ -9066,98 +7136,6 @@
 If you want, I can also provide a **one-page STM32CubeU3 migration checklist template** you can reuse for future package upgrades.</t>
   </si>
   <si>
-    <t>On STM32CubeU3, I2C sometimes gets stuck BUSY after a communication error and the bus never recovers. What is a safe software recovery sequence without full MCU reset?</t>
-  </si>
-  <si>
-    <t>A safe recovery is usually a **bus-unfreeze + peripheral re-init** sequence:
-## Recommended recovery flow
-1. **Abort the current I2C activity**
-   - Stop any ongoing transfer/IT/DMA.
-   - Disable I2C interrupts and DMA requests.
-   - Clear pending I2C error/status flags as applicable in your HAL/LL flow.
-2. **Disable the I2C peripheral**
-   - This releases control of the pins and lets you manipulate them as GPIO if needed.
-3. **Recover the bus at GPIO level**
-   If **SDA is stuck low** or **BUSY never clears**, try to free the slave by clocking SCL manually:
-   - Reconfigure **SCL and SDA as GPIO open-drain outputs** with pull-ups.
-   - Drive **SCL high/low up to 9 pulses** while monitoring SDA.
-   - If SDA is released, generate a **STOP condition** manually:
-     - SDA low while SCL high
-     - then SDA high while SCL high
-4. **Optionally reset the I2C peripheral block**
-   - Use the peripheral reset in RCC if available for your instance.
-   - This is not a full MCU reset, only the I2C domain.
-5. **Restore I2C pin alternate function**
-   - Reconfigure SCL/SDA back to I2C AF open-drain.
-6. **Reinitialize the I2C peripheral**
-   - Call your normal `MX_I2Cx_Init()` / `HAL_I2C_Init()`.
-   - Clear/refresh state variables if using HAL handle-based state machine.
-7. **Retry the transaction**
-   - Prefer a bounded retry count and a timeout.
----
-## Practical STM32 HAL-style sequence
-Typical safe order:
-```c
-HAL_I2C_DeInit(&amp;hi2c1);
-/* Optional: manually recover bus on GPIO if BUSY persists */
-I2C_BusRecover_GPIO();
-/* Re-init */
-HAL_I2C_Init(&amp;hi2c1);
-```
-If the bus is physically stuck, `HAL_I2C_DeInit()` alone is often **not enough**; the GPIO clocking step is the key part.
----
-## GPIO bus recovery idea
-```c
-static void I2C_BusRecover_GPIO(void)
-{
-    GPIO_InitTypeDef GPIO_InitStruct = {0};
-    /* 1) Disable I2C peripheral first */
-    /* 2) Configure SCL/SDA as open-drain GPIO */
-    GPIO_InitStruct.Pin = SCL_PIN | SDA_PIN;
-    GPIO_InitStruct.Mode = GPIO_MODE_OUTPUT_OD;
-    GPIO_InitStruct.Pull = GPIO_PULLUP;
-    GPIO_InitStruct.Speed = GPIO_SPEED_FREQ_LOW;
-    HAL_GPIO_Init(I2C_GPIO_PORT, &amp;GPIO_InitStruct);
-    HAL_GPIO_WritePin(I2C_GPIO_PORT, SCL_PIN | SDA_PIN, GPIO_PIN_SET);
-    HAL_Delay(1);
-    /* 3) Pulse SCL up to 9 times */
-    for (int i = 0; i &lt; 9; i++)
-    {
-        if (HAL_GPIO_ReadPin(I2C_GPIO_PORT, SDA_PIN) == GPIO_PIN_SET)
-            break;
-        HAL_GPIO_WritePin(I2C_GPIO_PORT, SCL_PIN, GPIO_PIN_RESET);
-        delay_us(5);
-        HAL_GPIO_WritePin(I2C_GPIO_PORT, SCL_PIN, GPIO_PIN_SET);
-        delay_us(5);
-    }
-    /* 4) Generate STOP if SDA is free */
-    if (HAL_GPIO_ReadPin(I2C_GPIO_PORT, SDA_PIN) == GPIO_PIN_SET)
-    {
-        HAL_GPIO_WritePin(I2C_GPIO_PORT, SDA_PIN, GPIO_PIN_RESET);
-        delay_us(5);
-        HAL_GPIO_WritePin(I2C_GPIO_PORT, SCL_PIN, GPIO_PIN_SET);
-        delay_us(5);
-        HAL_GPIO_WritePin(I2C_GPIO_PORT, SDA_PIN, GPIO_PIN_SET);
-        delay_us(5);
-    }
-}
-```
----
-## Notes specific to “BUSY stuck” cases
-- BUSY can remain set if the peripheral sampled a **false start/stop** or the bus is held low by a slave after an error.
-- On some STM32 families, a **peripheral reset** is the most reliable way to clear internal bus state.
-- If a slave is powered while the MCU I/O is not, the slave may **back-drive SDA/SCL**; GPIO pulsing will usually reveal this.
-- If your board lacks strong pull-ups or has a heavy bus capacitance, recovery pulses may need slower timing.
----
-## Best practice
-Use a layered recovery strategy:
-1. **Try `HAL_I2C_DeInit()` / peripheral reset**
-2. **If BUSY persists, do GPIO clock pulses + STOP**
-3. **Re-init I2C**
-4. **If still failing, isolate the offending slave or power-cycle that rail**
-If you want, I can provide a **STM32CubeU3-specific recovery function** using **HAL** or **LL**, ready to paste into your project.</t>
-  </si>
-  <si>
     <t>I need lower power consumption on STM32CubeU3 while preserving wake-up reliability. Which low-power configuration points should be audited first (clocks, GPIO state, peripherals, wake-up sources)?</t>
   </si>
   <si>
@@ -9550,120 +7528,6 @@
 If you want, I can also give you a **peripheral-specific migration checklist** for **USART / I2C / SPI / ADC / TIM / LPTIM / DMA / RTC** on STM32U5.</t>
   </si>
   <si>
-    <t>On STM32CubeU5, I2C sometimes gets stuck BUSY after a communication error and the bus never recovers. What is a safe software recovery sequence without full MCU reset?</t>
-  </si>
-  <si>
-    <t>Yes — on STM32U5 I2C, a stuck **BUSY** after an error is typically recovered by doing a **software peripheral recovery** plus a **bus unwedging** sequence if the lines are not idle.
-## Safe recovery sequence
-### 1) Stop using the I2C peripheral immediately
-Abort any ongoing transfer and disable I2C.
-- If using **HAL**, first abort the ongoing transaction if possible:
-  - `HAL_I2C_Master_Abort_IT()`
-  - or `HAL_I2C_DeInit()` if the handle is no longer reliable
-- Then disable the peripheral:
-  - clear `PE` bit in `I2C_CR1`
-### 2) Check the physical bus lines
-Read the GPIO levels for:
-- **SCL**
-- **SDA**
-If either line is held low, the bus is not electrically idle and the peripheral alone will not recover it.
-### 3) Reconfigure I2C pins as GPIO open-drain
-Temporarily switch SCL and SDA from I2C AF to:
-- **GPIO output open-drain**
-- with pull-up enabled externally or internally if necessary
-This allows you to manually generate clocks.
-### 4) Generate recovery clock pulses on SCL
-Pulse **SCL** up to **9 times** while monitoring **SDA**.
-Purpose: release a slave that is holding SDA low waiting for more clock edges.
-Typical behavior:
-- Drive SCL low
-- Release SCL high
-- Repeat up to 9 times
-- Stop early if SDA is released high
-### 5) Generate a STOP condition manually
-After SDA is released:
-- Ensure SCL is high
-- Drive SDA low
-- Then release SDA high while SCL remains high
-This recreates a bus STOP and helps reset slave state machines.
-### 6) Restore I2C pin alternate function
-Reconfigure pins back to I2C AF mode and reinitialize the peripheral.
-Recommended:
-- `HAL_I2C_DeInit()`
-- `HAL_I2C_Init()`
-If needed, also reset the peripheral registers by toggling the I2C kernel reset in RCC if software deinit is insufficient.
----
-## Recommended recovery order
-```text
-Abort transfer
-→ Disable I2C peripheral
-→ Check SCL/SDA GPIO state
-→ If SDA low: pulse SCL up to 9 times
-→ Generate STOP
-→ Restore AF mode
-→ Reinitialize I2C
-→ Retry transaction
-```
----
-## Practical STM32Cube/HAL approach
-A robust sequence is:
-1. `HAL_I2C_DeInit(&amp;hi2c);`
-2. Reconfigure SCL/SDA as GPIO open-drain
-3. Clock SCL manually until SDA is released
-4. Generate STOP
-5. Reconfigure pins to I2C AF
-6. `HAL_I2C_Init(&amp;hi2c);`
-If the peripheral remains stuck even after line recovery, add an **I2C peripheral reset** through RCC:
-- enable peripheral reset
-- then release reset
-- re-init I2C
----
-## Important cautions
-- Do **not** toggle SCL/SDA as push-pull outputs.
-- Avoid recovery while another master is active on the bus.
-- If a slave is truly wedged because of its own internal fault, it may need a device-specific reset or power-cycle.
-- If **SCL** is held low by a slave, software recovery may not work; that usually indicates a hardware fault or a slave stretching forever.
----
-## Minimal recovery pseudo-code
-```c
-void I2C_BusRecover(void)
-{
-    // 1. Disable I2C
-    __HAL_I2C_DISABLE(&amp;hi2c1);
-    // 2. Switch pins to GPIO open-drain
-    I2C_GPIO_RecoverMode();
-    // 3. If SDA low, pulse SCL up to 9 times
-    for (int i = 0; i &lt; 9 &amp;&amp; SDA_READ() == 0; i++)
-    {
-        SCL_LOW();
-        delay_us(5);
-        SCL_HIGH();
-        delay_us(5);
-    }
-    // 4. Generate STOP
-    SDA_LOW();
-    delay_us(5);
-    SCL_HIGH();
-    delay_us(5);
-    SDA_HIGH();
-    delay_us(5);
-    // 5. Restore I2C AF mode
-    I2C_GPIO_AFMode();
-    // 6. Re-init peripheral
-    HAL_I2C_Init(&amp;hi2c1);
-}
-```
----
-## Best practice on STM32U5
-If you want the most reliable solution, implement a **bus recovery state machine**:
-- error callback sets a recovery flag
-- main loop or task performs recovery
-- transaction is retried only after bus idle is confirmed
-If you want, I can provide:
-- a **STM32CubeU5 HAL-ready recovery function**
-- or a **LL/register-level version** for a specific I2C instance like `I2C1` or `I2C3`.</t>
-  </si>
-  <si>
     <t>I need lower power consumption on STM32CubeU5 while preserving wake-up reliability. Which low-power configuration points should be audited first (clocks, GPIO state, peripherals, wake-up sources)?</t>
   </si>
   <si>
@@ -9770,603 +7634,6 @@
 If you want, I can also give you a **STM32CubeU5 low-power checklist mapped to CubeMX settings and HAL APIs** for **Sleep / Stop / Standby** modes.</t>
   </si>
   <si>
-    <t>My STM32CubeWB project crashes with HardFault when enabling DMA in interrupt mode. Polling mode works. What should I verify first in clock, memory alignment, and interrupt configuration?</t>
-  </si>
-  <si>
-    <t>Here’s the **first checklist** I would verify when **DMA works in polling mode but HardFaults in interrupt mode** on **STM32CubeWB**:
----
-## 1) Clock configuration: make sure the DMA and peripheral clocks are really enabled
-Verify that:
-- The **DMA controller clock** is enabled in `MX_DMA_Init()` or equivalent.
-- The **peripheral clock** for the DMA-linked IP is enabled **before** starting the transfer.
-- If the DMA request comes from a peripheral with its own clock domain, that clock is also active.
-### What to check
-- `__HAL_RCC_DMA1_CLK_ENABLE()` or the correct DMA clock enable macro.
-- Peripheral clock enable call happens **before** `HAL_DMA_Start_IT()` / `HAL_UART_Receive_DMA()` / etc.
-- No low-power or clock reconfiguration disables the clock during the transfer.
-### Typical symptom
-If the DMA clock is not enabled, the first register access in interrupt-driven flow can lead to a fault or silent failure.
----
-## 2) Memory alignment and buffer location: ensure DMA-safe memory
-DMA is sensitive to:
-- **Alignment**
-- **Address validity**
-- **Buffer lifetime**
-- **Memory region accessibility**
-### Verify buffer rules
-- The DMA buffer is **not on the stack** if it may be used after the function returns.
-- The buffer is placed in **RAM accessible by DMA**.
-- The buffer is properly aligned for the data width.
-### Check alignment example
-If using 16-bit transfers, the buffer should be at least 2-byte aligned.  
-For 32-bit transfers, 4-byte alignment is safer.
-### Also verify
-- Source/destination pointers are valid and not `NULL`.
-- Length matches the buffer size and transfer width.
-- The buffer is not declared `const` if DMA writes into it.
-### Example
-```c
-__attribute__((aligned(4))) uint8_t rxBuffer[128];
-```
----
-## 3) Interrupt configuration: DMA IRQ must be enabled and linked correctly
-Polling mode does not need interrupts, so this is a common reason why interrupt mode fails.
-### Verify:
-- The **DMA IRQ line** is enabled in NVIC.
-- The **IRQ handler** calls `HAL_DMA_IRQHandler()` for the correct DMA handle.
-- The DMA handle is correctly linked to the peripheral handle.
-### Typical checks
-```c
-HAL_NVIC_SetPriority(DMA1_Channel1_IRQn, 0, 0);
-HAL_NVIC_EnableIRQ(DMA1_Channel1_IRQn);
-```
-And in the IRQ handler:
-```c
-void DMA1_Channel1_IRQHandler(void)
-{
-  HAL_DMA_IRQHandler(&amp;hdma_xxx);
-}
-```
-### Also check
-- The correct interrupt name for your exact DMA channel/request.
-- No conflicting handler or missing callback registration.
-- Priority is not blocked by another higher-priority interrupt forever.
----
-## 4) Confirm the DMA handle / callback linkage
-Make sure the peripheral is linked to the DMA handle properly:
-```c
-__HAL_LINKDMA(&amp;hperiph, hdmarx, hdma_xxx);
-```
-If this is wrong or missing, the HAL interrupt path may dereference invalid handles and fault.
----
-## 5) If using cache or special memory regions, review memory attributes
-On some STM32 families this matters a lot, but for STM32WB it is still worth verifying:
-- Buffer is in a region that is **DMA-accessible**
-- No invalid MPU settings
-- No corrupted stack/heap usage
----
-## 6) Look at the HardFault cause register values
-If possible, inspect:
-- `CFSR`
-- `HFSR`
-- `BFAR`
-- `MMFAR`
-This tells you whether the fault is due to:
-- invalid memory access
-- bus fault during ISR
-- unaligned access
-- bad pointer in HAL callback path
----
-## Recommended first order of investigation
-1. **DMA clock enabled**
-2. **Peripheral clock enabled**
-3. **Buffer address/alignment and lifetime**
-4. **NVIC IRQ enabled**
-5. **IRQ handler calls `HAL_DMA_IRQHandler()`**
-6. **DMA handle linked with `__HAL_LINKDMA()`**
----
-## Fast practical test
-If polling works, try this minimal interrupt-mode test:
-- Use a **global static buffer**
-- Confirm **DMA clock + peripheral clock**
-- Enable the **exact DMA IRQ**
-- Put a breakpoint in the DMA ISR
-- Confirm the ISR is entered and `HAL_DMA_IRQHandler()` is executed
----
-If you want, I can give you a **STM32WB-specific DMA interrupt-mode checklist** or help you inspect your **`MX_DMA_Init()`**, **IRQ handler**, and **HardFault registers** line by line.</t>
-  </si>
-  <si>
-    <t>WB</t>
-  </si>
-  <si>
-    <t>After updating to a newer STM32CubeWB package release, a previously working peripheral init now fails. What is the best migration/debug checklist to identify breaking changes quickly?</t>
-  </si>
-  <si>
-    <t>## Fast migration/debug checklist for STM32CubeWB package updates
-When a peripheral initialization breaks after a CubeWB package update, the fastest way to isolate the regression is to **separate user code, generated code, middleware, and low-level configuration changes**. Here is a practical checklist.
----
-### 1) Confirm the exact package delta
-- Note the **old** and **new** STM32CubeWB versions
-- Read the **Release Notes / Migration Notes** for both:
-  - HAL/LL API changes
-  - middleware changes
-  - board support package updates
-  - known issues and fixed bugs
-- Search specifically for your peripheral name and any related middleware
-**Goal:** determine whether the failure is due to an API change, a default configuration change, or a bug fix that exposed a latent issue.
----
-### 2) Diff the generated project files
-Compare the old working project and the newly generated one:
-- `Core/Inc/*`
-- `Core/Src/*`
-- `Drivers/STM32WBxx_HAL_Driver/*` if you copied or modified them locally
-- `Middlewares/*`
-- `STM32WB*.ioc`
-- startup and linker files if relevant
-Focus on:
-- `MX_&lt;PERIPH&gt;_Init()`
-- `HAL_&lt;PERIPH&gt;_Init()`
-- `HAL_&lt;PERIPH&gt;_MspInit()`
-- clock tree setup
-- IRQ priorities and NVIC enables
-- GPIO alternate-function configuration
-- DMA settings
-- peripheral instance selection
----
-### 3) Check for CubeMX regeneration overwriting assumptions
-A common issue is that regeneration changes:
-- pin assignments
-- peripheral clock source
-- prescaler values
-- GPIO speed/pull settings
-- middleware task ordering
-- initialization order
-Make sure:
-- **user code is only inside `/* USER CODE BEGIN */` blocks**
-- no manual edits were made in generated sections that got overwritten
-- the `.ioc` file still matches what you intended
----
-### 4) Verify clock configuration first
-Many peripheral init failures are clock-related.
-Check:
-- system clock source and frequency
-- peripheral clock source selection
-- AHB/APB prescalers
-- RF / low-speed clock dependencies if using wireless blocks or low-power features
-- RTC/LSE/LSI setup if the peripheral depends on timebase or wakeup behavior
-**Typical symptom:** `HAL_&lt;PERIPH&gt;_Init()` returns an error because the peripheral clock is not enabled or not at the expected source.
----
-### 5) Inspect `HAL_&lt;PERIPH&gt;_MspInit()` and `HAL_*_ClockConfig()`
-For many failures, the issue is in the MSP layer:
-- GPIO clocks enabled?
-- Peripheral clock enabled?
-- Correct alternate function assigned?
-- DMA channel/request updated?
-- IRQ enabled?
-- NVIC priority compatible with middleware?
-Also verify that deinit/init symmetry remains correct.
----
-### 6) Check for API signature or enum changes
-Search compile warnings and errors carefully for:
-- changed function parameters
-- renamed macros
-- deprecated definitions
-- enum value changes
-- structure field additions/reordering
-Even if it compiles, initialization may fail if:
-- default values changed
-- fields are no longer initialized as before
-- structure instances are partially initialized
-**Tip:** now compare all peripheral init structs using explicit initialization, not implicit defaults.
----
-### 7) Rebuild from clean state
-Do a full cleanup:
-- delete build output
-- regenerate code if needed
-- rebuild all
-This catches:
-- stale object files
-- old middleware headers
-- mixed-version driver artifacts
-If using IDE-managed builds, also clean the project metadata if the toolchain cache seems inconsistent.
----
-### 8) Instrument init return paths
-Add temporary checks:
-- print/log the return value of each init call
-- stop in debugger when a failure occurs
-- inspect `HAL_GetError()` if available
-- inspect peripheral state fields after init
-Example approach:
-- call each `MX_*_Init()` separately
-- place breakpoints before and after every `HAL_*_Init()`
-- verify which exact peripheral first fails
-**Goal:** identify whether the failure is in the peripheral itself or in something it depends on.
----
-### 9) Validate pin mux and hardware conflicts
-After Cube updates, pin mapping may shift due to board support or package changes.
-Check:
-- pins shared with debug, RF, oscillator, or user LEDs/buttons
-- wrong AF selection
-- conflicting use of the same pin by another peripheral
-- analog vs digital mode mismatch
-- external pull-ups/pull-downs assumptions
----
-### 10) Check middleware and wireless stack interactions
-For STM32WB specifically, middleware can affect peripheral startup:
-- BLE stack startup sequencing
-- CPU2 ownership of shared resources
-- IPCC, RTC, RNG, HW semaphores, low-power mode interactions
-- thread/RTOS initialization order if used
-If the failing peripheral is shared or timing-sensitive, try:
-- initializing it **before** middleware start
-- or **after** the wireless stack is fully up, depending on dependency
----
-### 11) Compare generated code to a fresh project of the new version
-Create a new empty project with the **same board and peripheral selection** in the new CubeWB version, then compare:
-- generated init code
-- clock config
-- MSP code
-- middleware setup
-This is often the fastest way to identify:
-- changed defaults
-- required new settings
-- generator behavior changes
----
-### 12) Bisect the problem
-If the regression source is not obvious:
-- revert one change at a time between versions
-- isolate one peripheral at a time
-- disable middleware temporarily
-- reduce to a minimal init example
-This helps distinguish:
-- package migration issue
-- project configuration issue
-- hardware issue surfaced by tighter validation
----
-## Practical debug order
-If you want the quickest path, use this order:
-1. **Check release notes**
-2. **Diff generated init + clock + MSP files**
-3. **Verify peripheral clocks and GPIO AF**
-4. **Clean rebuild**
-5. **Instrument every init call**
-6. **Compare with a fresh project in the new CubeWB version**
-7. **Isolate middleware interaction**
----
-## Common causes after Cube updates
-- peripheral clock source changed
-- new default GPIO speed/pull settings
-- DMA request/channel mapping changed
-- init order changed
-- middleware now requires an extra clock or semaphore setup
-- a previously tolerated configuration is now rejected by the HAL
-- stale generated files from mixed package versions
----
-## Recommended workflow for future upgrades
-- keep the old working project as a reference branch
-- regenerate a new project in the target CubeWB version
-- diff only the generated sections
-- migrate user code incrementally
-- validate one peripheral at a time
----
-If you want, I can also provide:
-1. a **one-page STM32CubeWB migration checklist template**, or  
-2. a **debug script/logging snippet** to pinpoint which `HAL_*_Init()` is failing.</t>
-  </si>
-  <si>
-    <t>On STM32CubeWB, I2C sometimes gets stuck BUSY after a communication error and the bus never recovers. What is a safe software recovery sequence without full MCU reset?</t>
-  </si>
-  <si>
-    <t>A safe and commonly used **software-only I2C bus recovery** on **STM32CubeWB** is:
-1. **Stop the I2C peripheral**
-2. **Release the pins from alternate-function I2C**
-3. **Manually toggle SCL to free a stuck slave**
-4. **Generate a STOP condition if possible**
-5. **Re-initialize the peripheral**
-6. **Clear HAL/I2C error state**
-7. **Restart communication**
-This is the typical approach when `BUSY` remains set after an error and the bus is likely held by a slave waiting for clocks.
----
-## Recommended recovery sequence
-### 1) Abort/disable the I2C peripheral
-If a transfer is ongoing or the peripheral is in an error state:
-```c
-HAL_I2C_DeInit(&amp;hi2c1);
-```
-If the peripheral does not deinit cleanly, force-disable it via registers before reconfiguring pins.
----
-### 2) Reconfigure SCL and SDA as GPIO open-drain
-Set both lines temporarily as GPIO outputs open-drain with pull-up, then release them high.
-- **SDA = input/open-drain high**
-- **SCL = open-drain high**
-This lets you inspect the actual line levels and manually recover the bus.
----
-### 3) Clock out a stuck slave
-If **SDA is low**, a slave may be waiting for more clock pulses. Toggle **SCL** up to **9 pulses** while monitoring SDA:
-- Drive SCL low
-- Release SCL high
-- Repeat up to 9 times
-- Stop early if SDA is released high
-This is the standard method to flush a slave stuck mid-byte.
-Pseudo-code:
-```c
-static void I2C_BusRecovery(GPIO_TypeDef *SCL_Port, uint16_t SCL_Pin,
-                            GPIO_TypeDef *SDA_Port, uint16_t SDA_Pin)
-{
-    GPIO_InitTypeDef GPIO_InitStruct = {0};
-    __HAL_RCC_GPIOB_CLK_ENABLE(); // adjust to your port
-    // Configure SCL/SDA as open-drain outputs
-    GPIO_InitStruct.Pin = SCL_Pin | SDA_Pin;
-    GPIO_InitStruct.Mode = GPIO_MODE_OUTPUT_OD;
-    GPIO_InitStruct.Pull = GPIO_PULLUP;
-    GPIO_InitStruct.Speed = GPIO_SPEED_FREQ_HIGH;
-    HAL_GPIO_Init(SCL_Port, &amp;GPIO_InitStruct);
-    HAL_GPIO_WritePin(SCL_Port, SCL_Pin | SDA_Pin, GPIO_PIN_SET);
-    HAL_Delay(1);
-    // If SDA is low, generate clocks on SCL
-    if (HAL_GPIO_ReadPin(SDA_Port, SDA_Pin) == GPIO_PIN_RESET)
-    {
-        for (int i = 0; i &lt; 9; i++)
-        {
-            HAL_GPIO_WritePin(SCL_Port, SCL_Pin, GPIO_PIN_RESET);
-            HAL_Delay(1);
-            HAL_GPIO_WritePin(SCL_Port, SCL_Pin, GPIO_PIN_SET);
-            HAL_Delay(1);
-            if (HAL_GPIO_ReadPin(SDA_Port, SDA_Pin) == GPIO_PIN_SET)
-                break;
-        }
-    }
-    // Generate a STOP condition:
-    // SDA low while SCL high, then SDA high
-    HAL_GPIO_WritePin(SCL_Port, SCL_Pin, GPIO_PIN_RESET);
-    HAL_Delay(1);
-    HAL_GPIO_WritePin(SDA_Port, SDA_Pin, GPIO_PIN_RESET);
-    HAL_Delay(1);
-    HAL_GPIO_WritePin(SCL_Port, SCL_Pin, GPIO_PIN_SET);
-    HAL_Delay(1);
-    HAL_GPIO_WritePin(SDA_Port, SDA_Pin, GPIO_PIN_SET);
-    HAL_Delay(1);
-}
-```
----
-### 4) Restore I2C alternate function
-After the bus is released:
-```c
-HAL_I2C_Init(&amp;hi2c1);
-```
-If you use MSP init code generated by CubeMX, make sure the GPIOs are put back to the proper **I2C AF open-drain** pins.
----
-### 5) Clear HAL state and error flags
-Before restarting, clear the HAL handle state so the driver does not remain locked in error:
-```c
-hi2c1.ErrorCode = HAL_I2C_ERROR_NONE;
-hi2c1.State = HAL_I2C_STATE_READY;
-```
-If your application uses timeouts and callbacks, also ensure no transfer is still marked active.
----
-## Safer complete recovery helper
-A robust pattern is:
-```c
-void I2C1_Recover(I2C_HandleTypeDef *hi2c)
-{
-    HAL_I2C_DeInit(hi2c);
-    I2C_BusRecovery(SCL_GPIO_Port, SCL_Pin, SDA_GPIO_Port, SDA_Pin);
-    HAL_I2C_Init(hi2c);
-    hi2c-&gt;ErrorCode = HAL_I2C_ERROR_NONE;
-    hi2c-&gt;State = HAL_I2C_STATE_READY;
-}
-```
----
-## Important notes
-- **Do not recover the bus while another master may still be active.**
-- If **SCL is held low** by a slave, GPIO clock pulsing will not help; you can only recover if the slave can release SCL or if the stuck condition is internal to the MCU/peripheral.
-- For **I2C v2/v3 peripherals** on STM32, a peripheral reset may sometimes be needed if `BUSY` is internal and the pins are actually free.
-- After an error like **AF** or **BERR**, it is often better to:
-  - disable the peripheral,
-  - clear error conditions,
-  - reconfigure pins,
-  - re-enable I2C.
----
-## Practical recommendation for STM32CubeWB
-For STM32WB projects, the most reliable sequence is:
-1. `HAL_I2C_DeInit()`
-2. GPIO recovery on SCL/SDA
-3. `HAL_I2C_Init()`
-4. Reset `hi2c-&gt;ErrorCode` and `hi2c-&gt;State`
-5. Retry transaction with a limit
----
-If you want, I can provide a **CubeWB-ready recovery function** tailored to your exact I2C instance and pin mapping.</t>
-  </si>
-  <si>
-    <t>I need lower power consumption on STM32CubeWB while preserving wake-up reliability. Which low-power configuration points should be audited first (clocks, GPIO state, peripherals, wake-up sources)?</t>
-  </si>
-  <si>
-    <t>## Low-power audit checklist for STM32CubeWB
-If your goal is **lower consumption without hurting wake-up reliability**, I’d audit these areas first, in this order:
-### 1) **Clock tree and runtime clock switching**
-Verify that the system really drops to the expected low-power clocking scheme before sleep/stop.
-**Audit points**
-- **No high-speed clock left running** unnecessarily:
-  - HSE / HSI16 / PLL off in low-power entry, unless explicitly needed.
-  - On STM32WB, confirm the CPU is not kept on a boosted clock path by software.
-- **System clock source after wake-up** is restored correctly:
-  - Ensure `SystemClock_Config()` is called appropriately after Stop/Standby exit if needed.
-- **Peripheral clock gating**:
-  - Disable unused peripheral clocks in RCC before entering low power.
-- **MCO outputs**:
-  - Make sure `MCO` pins are disabled if used during debug or test.
-- **Radio/BLE stack timing**:
-  - For WB, check that the wireless stack is not forcing frequent wakeups or keeping time bases active.
-**What to measure**
-- Current draw before sleep, in sleep/stop, and immediately after wake-up.
-- Oscilloscope/logic analyzer on a GPIO toggled around low-power entry/exit to confirm actual residency.
----
-### 2) **GPIO state and leakage paths**
-GPIO misconfiguration is one of the most common causes of excess current.
-**Audit points**
-- **Unused pins**:
-  - Set to **Analog mode** with **no pull** when possible.
-  - Avoid floating inputs.
-- **External circuitry interaction**:
-  - Check pins connected to sensors, LEDs, level shifters, pull-ups, and transceivers.
-  - A pin left driving an external device can dominate power.
-- **Output levels before stop**:
-  - Drive pins to a safe static level before entering low power to avoid shoot-through or leakage.
-- **Wake-up pins**:
-  - Ensure wake pins have the proper pull configuration and are not floating.
-- **Debug pins**:
-  - SWD/JTAG pins can keep parts alive or leak current depending on board configuration.
-**Very common issues**
-- LED GPIOs not turned off.
-- External pull-ups too strong on wake lines.
-- Alternate-function pins left active even though the peripheral is disabled.
----
-### 3) **Peripheral shutdown and hidden activity**
-Even if the CPU sleeps, peripherals can keep consuming power or generate wake events.
-**Audit points**
-- **UART, SPI, I2C, ADC, timers, DMA**:
-  - Disable peripherals that are not needed.
-  - Stop ongoing DMA transfers before entering low power.
-- **Timers/time bases**:
-  - SysTick or HAL tick may keep waking the core.
-  - Confirm the tick is suspended when entering Stop mode if appropriate.
-- **Middleware activity**:
-  - BLE, thread, or other middleware may schedule periodic wake-ups.
-  - Check whether any task/event loop prevents deep sleep.
-- **IRQ sources left enabled**:
-  - Unused interrupts should be masked to prevent spurious wakeups.
-- **Analog peripherals**:
-  - ADC, comparator, OPAMP, VREFBUF, and internal pull networks may need explicit disable.
-**WB-specific note**
-- The wireless subsystem may have its own low-power constraints and wake scheduling. Make sure the application aligns with the stack’s power policy.
----
-### 4) **Wake-up sources and their electrical integrity**
-To preserve reliability, wake-up sources must be configured carefully, not merely enabled.
-**Audit points**
-- **Correct selection of wake source**:
-  - EXTI line, RTC alarm, RTC wakeup timer, radio event, GPIO wake pin, etc.
-- **Edge polarity and filtering**:
-  - Verify rising/falling edge matches the actual signal behavior.
-  - Add hardware or software debounce if needed.
-- **Signal idle state**:
-  - Ensure the wake signal sits at a valid level during sleep, not floating.
-- **Race conditions on entry/exit**:
-  - Clear pending EXTI/RTC flags *before* entering sleep.
-  - Confirm no stale interrupt is immediately retriggering wake.
-- **Clock domain dependency**:
-  - Some wake sources require specific clocking or LSE/LSI validity.
-  - Confirm RTC uses a stable low-speed clock source.
-- **Button wake reliability**:
-  - For mechanical buttons, add debounce and consider EMI susceptibility.
-**Practical check**
-- Wake from each source individually, many times, across temperature and supply range if possible.
----
-## Recommended first-pass audit order
-1. **GPIO unused pins and external leakage**
-2. **High-speed clocks / PLL / peripheral clock gating**
-3. **SysTick, timers, DMA, and middleware periodic activity**
-4. **Wake-up source configuration and pending flags**
-5. **WB wireless stack power-policy interactions**
----
-## Quick STM32CubeWB checklist
-- `GPIOx` unused pins → **Analog**
-- Disable **PLL/HSE/HSI16** before Stop if allowed
-- Suspend **HAL tick** in Stop mode when appropriate
-- Disable unused **peripheral clocks**
-- Clear **pending EXTI/RTC flags**
-- Verify **RTC clock source** and wake timer behavior
-- Check **debug/SWD** influence on current
-- Confirm the **BLE/wireless stack** isn’t scheduling frequent wakeups
----
-## Best debugging approach
-If you want reliability **and** low current, test in this sequence:
-1. **Measure baseline current** with only MCU + board.
-2. **Force all unused GPIO to analog**.
-3. **Disable all nonessential peripherals**.
-4. **Enter Stop mode with one known wake source**.
-5. **Add back wake sources one by one** and verify current and wake success.
-6. **Finally enable middleware / wireless features** and re-check.
-If you want, I can give you a **CubeMX/CubeWB audit checklist** or a **code-level low-power template for STM32WB Stop mode**.</t>
-  </si>
-  <si>
-    <t>My STM32CubeWB0 project crashes with HardFault when enabling DMA in interrupt mode. Polling mode works. What should I verify first in clock, memory alignment, and interrupt configuration?</t>
-  </si>
-  <si>
-    <t>Here’s the **first checklist** I would verify for a **HardFault that appears only when DMA interrupt mode is enabled** on **STM32CubeWB0**.
-## 1) Clock configuration
-Verify that the DMA and peripheral clocks are **actually enabled before starting DMA**:
-- **DMA clock enabled**
-  - Check the corresponding `__HAL_RCC_xxx_CLK_ENABLE()` call for the DMA controller used by your peripheral.
-- **Peripheral clock enabled**
-  - The source peripheral must have its clock enabled before DMA starts.
-- **NVIC clock-independent?**
-  - NVIC does not need a clock, but the **peripheral IRQ must be enabled** and prioritized correctly.
-Also confirm:
-- The selected **system clock source is stable**
-- Any low-power clock or MSI/HSI configuration is not changing during the transfer
-- If the DMA request comes from a peripheral with a specific clock domain, that domain is up and running
-## 2) Memory alignment and buffer validity
-HardFaults in interrupt DMA mode often come from **invalid or misaligned buffers**.
-Check:
-- The DMA buffer is:
-  - **global or static**, not a local stack variable that goes out of scope
-  - **properly aligned** for the transfer width
-- The buffer address is valid and accessible by DMA
-- The buffer size matches the transfer length exactly
-- The source/destination pointer is not `NULL`
-- The buffer is not in a memory region inaccessible to DMA
-### Alignment rules to verify
-If DMA transfers:
-- **byte** data: usually no special alignment
-- **half-word** data: buffer should be aligned to 2 bytes
-- **word** data: buffer should be aligned to 4 bytes
-If cache is involved on your device/variant, also verify cache maintenance. On **WB0**, cache issues are usually less central than on larger Cortex-M7 parts, but buffer placement and alignment still matter.
-## 3) Interrupt configuration
-Interrupt mode adds one very common failure point: **IRQ setup**.
-Verify:
-- The DMA IRQ handler is present in `stm32wb0xx_it.c`
-- The handler calls the HAL IRQ handler, for example:
-  - `HAL_DMA_IRQHandler(&amp;hdma_xxx);`
-- The IRQ is enabled in NVIC:
-  - `HAL_NVIC_EnableIRQ(...)`
-- Priority is valid and not too high/low for your system setup
-- The DMA callback pointers are correctly linked to the peripheral handle
-  - e.g. `__HAL_LINKDMA(...)`
-## 4) HAL handle linkage
-Make sure the peripheral handle and DMA handle are properly connected:
-- `hdma.Instance` is correct
-- `hdma.Init.Request` matches the peripheral DMA request
-- `__HAL_LINKDMA(&amp;hperiph, hdmatx, hdma_tx)` or `hdmarx` is done
-- The peripheral is initialized **after** DMA configuration if required by the HAL sequence
-## 5) Common “works in polling, fails in interrupt” causes
-This pattern usually points to one of these:
-- Missing `HAL_NVIC_EnableIRQ()`
-- Missing `HAL_DMA_IRQHandler()`
-- DMA handle not linked with `__HAL_LINKDMA()`
-- Buffer allocated on the stack
-- Wrong buffer alignment
-- Interrupt fires before the handle is fully initialized
-- Wrong DMA request/channel selection
-- Overrun due to a too-fast interrupt source or bad length
-## 6) Fast debug approach
-Try this order:
-1. Confirm **DMA clock enabled**
-2. Confirm **buffer is static/global and aligned**
-3. Confirm **IRQ handler calls HAL handler**
-4. Confirm **NVIC IRQ enabled**
-5. Confirm **DMA handle linked to peripheral handle**
-6. Confirm **transfer length and data width match**
-## 7) Recommended trace points
-Put breakpoints or logs at:
-- DMA init completion
-- `HAL_DMA_Start_IT(...)` or equivalent
-- DMA IRQ entry
-- `HAL_DMA_IRQHandler(...)`
-- HAL transfer-complete / error callbacks
-- `HardFault_Handler`
-If you want, I can help you build a **WB0-specific checklist** for your exact peripheral, such as **USART, SPI, ADC, I2C, or TIM** DMA interrupt mode.</t>
-  </si>
-  <si>
     <t>WB0</t>
   </si>
   <si>
@@ -10545,126 +7812,6 @@
 - **Release note breaking changes**
 ---
 If you want, I can also provide a **migration checklist template** tailored to a specific peripheral such as **UART, I2C, SPI, ADC, TIM, or RTC**.</t>
-  </si>
-  <si>
-    <t>On STM32CubeWB0, I2C sometimes gets stuck BUSY after a communication error and the bus never recovers. What is a safe software recovery sequence without full MCU reset?</t>
-  </si>
-  <si>
-    <t>A safe recovery for a stuck **I2C BUSY** on **STM32CubeWB0** is to **fully deinitialize the peripheral, force clocked GPIO bus-unwedge pulses on SCL, generate a STOP if possible, then reinitialize I2C**. This avoids a full MCU reset and is commonly used when a slave holds **SDA low** after a communication error.
-## Recommended recovery sequence
-### 1) Disable I2C and clear its state
-- Disable I2C peripheral.
-- Clear pending error flags / stop any ongoing transfer.
-- Abort any HAL transfer state if needed.
-Typical idea:
-```c
-HAL_I2C_DeInit(&amp;hi2c1);
-```
-If you use interrupts/DMA, also stop them first:
-```c
-HAL_I2C_Master_Abort_IT(&amp;hi2c1, dev_addr);
-```
-or abort DMA paths as applicable.
----
-### 2) Reconfigure SCL and SDA as GPIO open-drain
-- Switch both pins to **GPIO output open-drain**.
-- Enable pull-ups if your board does not already provide strong ones.
-- Set both lines **high** initially.
-This ensures you can manually toggle SCL without fighting the peripheral.
----
-### 3) Clock out up to 9 pulses on SCL
-- If a slave is stuck mid-byte, it may release SDA after seeing enough SCL edges.
-- Generate **9 SCL pulses** minimum.
-- Keep SDA released/high during the pulses.
-Pseudo-sequence:
-1. SCL low
-2. SCL high
-3. repeat 9 times
----
-### 4) Try to generate a STOP condition manually
-After the pulses:
-- Drive **SDA low**
-- Release **SCL high**
-- Then release **SDA high**
-This emulates a STOP and often clears the slave state machine.
----
-### 5) Check bus idle
-Verify:
-- **SCL = 1**
-- **SDA = 1**
-If either line is still low:
-- The slave may still be holding the bus, or there may be a hardware fault.
-- You can retry the pulse sequence once or twice.
-- If it still fails, a power-cycle of the slave may be required.
----
-### 6) Reinitialize the I2C peripheral
-Once the bus is idle again:
-```c
-HAL_I2C_Init(&amp;hi2c1);
-```
-Then restore DMA/IRQ config if used.
----
-## Practical safe recovery function skeleton
-```c
-void I2C_BusRecovery(void)
-{
-    GPIO_InitTypeDef GPIO_InitStruct = {0};
-    /* 1. Deinit I2C */
-    HAL_I2C_DeInit(&amp;hi2c1);
-    /* 2. Configure SCL/SDA as GPIO open-drain */
-    __HAL_RCC_GPIOB_CLK_ENABLE();   // example port
-    GPIO_InitStruct.Pin = I2C_SCL_Pin | I2C_SDA_Pin;
-    GPIO_InitStruct.Mode = GPIO_MODE_OUTPUT_OD;
-    GPIO_InitStruct.Pull = GPIO_PULLUP;
-    GPIO_InitStruct.Speed = GPIO_SPEED_FREQ_HIGH;
-    HAL_GPIO_Init(I2C_SCL_GPIO_Port, &amp;GPIO_InitStruct);
-    /* Release both lines */
-    HAL_GPIO_WritePin(I2C_SCL_GPIO_Port, I2C_SCL_Pin | I2C_SDA_Pin, GPIO_PIN_SET);
-    HAL_Delay(1);
-    /* 3. Clock SCL 9 times */
-    for (int i = 0; i &lt; 9; i++)
-    {
-        HAL_GPIO_WritePin(I2C_SCL_GPIO_Port, I2C_SCL_Pin, GPIO_PIN_RESET);
-        delay_us(5);
-        HAL_GPIO_WritePin(I2C_SCL_GPIO_Port, I2C_SCL_Pin, GPIO_PIN_SET);
-        delay_us(5);
-    }
-    /* 4. Manual STOP */
-    HAL_GPIO_WritePin(I2C_SCL_GPIO_Port, I2C_SCL_Pin, GPIO_PIN_SET);
-    delay_us(5);
-    HAL_GPIO_WritePin(I2C_SCL_GPIO_Port, I2C_SDA_Pin, GPIO_PIN_RESET);
-    delay_us(5);
-    HAL_GPIO_WritePin(I2C_SCL_GPIO_Port, I2C_SCL_Pin, GPIO_PIN_SET);
-    delay_us(5);
-    HAL_GPIO_WritePin(I2C_SCL_GPIO_Port, I2C_SDA_Pin, GPIO_PIN_SET);
-    delay_us(5);
-    /* 5. Optionally verify bus idle here */
-    if (HAL_GPIO_ReadPin(I2C_SCL_GPIO_Port, I2C_SCL_Pin) == GPIO_PIN_SET &amp;&amp;
-        HAL_GPIO_ReadPin(I2C_SDA_GPIO_Port, I2C_SDA_Pin) == GPIO_PIN_SET)
-    {
-        /* 6. Reinit I2C */
-        HAL_GPIO_DeInit(I2C_SCL_GPIO_Port, I2C_SCL_Pin | I2C_SDA_Pin);
-        HAL_I2C_Init(&amp;hi2c1);
-    }
-}
-```
----
-## Important notes for STM32WB0
-- Make sure the **I2C kernel clock** is valid after reinit.
-- If the peripheral reports **BUSY** because internal state is stuck, **deinit/init** is often enough only after the bus lines are physically released.
-- If the slave can be powered separately, a **slave reset or power-cycle** may be the only reliable last resort.
-- If another master exists on the bus, coordinate recovery to avoid collisions.
----
-## Best practice
-To improve robustness:
-- Enable **I2C error callbacks** and trigger recovery on:
-  - **BERR**
-  - **ARLO**
-  - **AF**
-  - **TIMEOUT**
-- Add a **bus-idle check** before every new transaction.
-- Use a **watchdog** to recover the system if the bus cannot be freed.
-If you want, I can also provide a **WB0-ready HAL recovery function** using your exact **SCL/SDA pin names and I2C instance**.</t>
   </si>
   <si>
     <t>I need lower power consumption on STM32CubeWB0 while preserving wake-up reliability. Which low-power configuration points should be audited first (clocks, GPIO state, peripherals, wake-up sources)?</t>
@@ -11041,71 +8188,6 @@
 If you want, I can also give you a **step-by-step STM32CubeWBA migration checklist template** you can use directly on a failing project.</t>
   </si>
   <si>
-    <t>On STM32CubeWBA, I2C sometimes gets stuck BUSY after a communication error and the bus never recovers. What is a safe software recovery sequence without full MCU reset?</t>
-  </si>
-  <si>
-    <t>A safe **software-only I2C bus recovery** on STM32CubeWBA is typically:
-## 1) Stop the peripheral first
-Disable the I2C peripheral and clear its error state so it no longer drives the lines:
-1. **Abort any ongoing transfer**
-2. **Disable I2C**
-3. **Clear I2C error flags**
-4. **Reconfigure GPIOs as open-drain outputs or inputs with pull-up**
-&gt; Goal: release control of **SCL/SDA** from the I2C peripheral before trying to free a slave that may be holding SDA low.
----
-## 2) Bit-bang the bus pulses on SCL
-If **SDA is stuck low**, generate up to **9 clock pulses on SCL** using GPIO:
-- Drive **SCL low**
-- Release **SCL high**
-- Wait for the line to actually go high
-- Repeat up to 9 times
-- Stop early if **SDA becomes high**
-This conventionally advances a slave out of a half-finished byte or ACK state.
----
-## 3) Generate a STOP condition manually
-After SDA is released:
-1. Ensure **SCL is high**
-2. Pull **SDA low**
-3. Release **SDA high** while **SCL remains high**
-This creates a valid **STOP**, which resets many slaves’ internal state machines.
----
-## 4) Restore I2C peripheral
-Then:
-1. Reconfigure pins back to **I2C alternate function open-drain**
-2. Re-enable the I2C peripheral
-3. Clear any remaining flags
-4. Reinitialize the hardware if needed
----
-## Recommended practical sequence
-A robust sequence is:
-1. `HAL_I2C_DeInit()`
-2. Configure **SCL/SDA as GPIO open-drain with pull-up**
-3. Check if **SDA low**
-4. Pulse **SCL up to 9 times**
-5. Generate **STOP**
-6. Return pins to I2C AF
-7. `HAL_I2C_Init()`
-8. Retry the transaction
----
-## Important safety notes
-- **Do not** reset the full MCU unless the bus still cannot be recovered.
-- Use **timeouts** on every wait for SCL/SDA transitions.
-- If another device is actively holding **SCL low**, software recovery may fail; in that case the slave may need its own reset or power-cycle.
-- If the WBA I2C peripheral itself is wedged, also perform a **peripheral reset via RCC** before reinit.
----
-## Minimal recovery logic
-```c
-// Pseudocode
-HAL_I2C_DeInit(&amp;hi2c1);
-// GPIO: SCL/SDA -&gt; open-drain outputs with pull-up
-I2C_BusRecover_PulseSCL_UpTo9();
-I2C_BusRecover_GenerateSTOP();
-// GPIO: back to AF I2C
-HAL_I2C_Init(&amp;hi2c1);
-```
-If you want, I can provide a **ready-to-use STM32CubeWBA C recovery function** for `HAL_I2C_MspDeInit()` / `HAL_I2C_MspInit()` style integration.</t>
-  </si>
-  <si>
     <t>I need lower power consumption on STM32CubeWBA while preserving wake-up reliability. Which low-power configuration points should be audited first (clocks, GPIO state, peripherals, wake-up sources)?</t>
   </si>
   <si>
@@ -11458,103 +8540,6 @@
 If you want, I can also give you a **targeted checklist for a specific peripheral** like **UART, I2C, SPI, ADC, RTC, SUBGHZ, or DMA**.</t>
   </si>
   <si>
-    <t>On STM32CubeWL, I2C sometimes gets stuck BUSY after a communication error and the bus never recovers. What is a safe software recovery sequence without full MCU reset?</t>
-  </si>
-  <si>
-    <t>A safe **software-only I2C bus recovery** on STM32CubeWL after a communication error usually follows this sequence:
-## 1) Stop any ongoing I2C activity
-- Abort the current transfer if needed.
-- Disable I2C peripheral so it no longer drives the bus.
-```c
-HAL_I2C_DeInit(&amp;hi2c1);
-```
-If the peripheral is not fully recoverable, you can also force-reset the I2C block via RCC reset:
-```c
-__HAL_RCC_I2C1_FORCE_RESET();
-__HAL_RCC_I2C1_RELEASE_RESET();
-```
-## 2) Switch SCL and SDA to GPIO open-drain
-Configure both pins as **GPIO output open-drain** with pull-up enabled, and release them high first.
-- SCL = GPIO open-drain output
-- SDA = GPIO open-drain output
-- Write both high
-This lets the master manually generate clock pulses.
-## 3) Clock the bus free
-If a slave is holding SDA low, generate up to **9 clock pulses** on SCL while monitoring SDA.
-Typical sequence:
-- Drive SCL low
-- Release SCL high
-- Repeat up to 9 times
-- Stop early if SDA becomes high
-This is the standard “unwedge” method for a slave stuck mid-byte.
-## 4) Generate a STOP condition manually
-Once SDA is released:
-- Ensure SCL is high
-- Pull SDA low
-- Release SDA high while SCL remains high
-This creates a STOP and returns the bus to idle.
-## 5) Reconfigure pins back to I2C
-Restore the pins to the I2C alternate-function open-drain configuration.
-## 6) Reinitialize I2C peripheral
-Call `HAL_I2C_Init()` again, or re-enable the peripheral after reset.
----
-# Recommended recovery function
-```c
-static HAL_StatusTypeDef I2C_BusRecovery(I2C_HandleTypeDef *hi2c)
-{
-    GPIO_InitTypeDef GPIO_InitStruct = {0};
-    // 1) Deinit I2C peripheral
-    HAL_I2C_DeInit(hi2c);
-    // 2) Configure SCL/SDA as GPIO open-drain outputs
-    // Replace with your actual ports/pins
-    GPIO_InitStruct.Pin = I2C1_SCL_PIN | I2C1_SDA_PIN;
-    GPIO_InitStruct.Mode = GPIO_MODE_OUTPUT_OD;
-    GPIO_InitStruct.Pull = GPIO_PULLUP;
-    GPIO_InitStruct.Speed = GPIO_SPEED_FREQ_HIGH;
-    HAL_GPIO_Init(I2C1_SCL_SDA_GPIO_PORT, &amp;GPIO_InitStruct);
-    // Release both lines high
-    HAL_GPIO_WritePin(I2C1_SCL_SDA_GPIO_PORT, I2C1_SCL_PIN | I2C1_SDA_PIN, GPIO_PIN_SET);
-    HAL_Delay(1);
-    // 3) Clock-out up to 9 pulses if SDA is held low
-    for (int i = 0; i &lt; 9 &amp;&amp; HAL_GPIO_ReadPin(I2C1_SCL_SDA_GPIO_PORT, I2C1_SDA_PIN) == GPIO_PIN_RESET; i++)
-    {
-        HAL_GPIO_WritePin(I2C1_SCL_SDA_GPIO_PORT, I2C1_SCL_PIN, GPIO_PIN_RESET);
-        HAL_Delay(1);
-        HAL_GPIO_WritePin(I2C1_SCL_SDA_GPIO_PORT, I2C1_SCL_PIN, GPIO_PIN_SET);
-        HAL_Delay(1);
-    }
-    // 4) Generate STOP condition: SDA low -&gt; SCL high -&gt; SDA high
-    HAL_GPIO_WritePin(I2C1_SCL_SDA_GPIO_PORT, I2C1_SDA_PIN, GPIO_PIN_RESET);
-    HAL_Delay(1);
-    HAL_GPIO_WritePin(I2C1_SCL_SDA_GPIO_PORT, I2C1_SCL_PIN, GPIO_PIN_SET);
-    HAL_Delay(1);
-    HAL_GPIO_WritePin(I2C1_SCL_SDA_GPIO_PORT, I2C1_SDA_PIN, GPIO_PIN_SET);
-    HAL_Delay(1);
-    // 5) Restore I2C AF mode
-    HAL_GPIO_DeInit(I2C1_SCL_SDA_GPIO_PORT, I2C1_SCL_PIN | I2C1_SDA_PIN);
-    // 6) Re-init I2C
-    return HAL_I2C_Init(hi2c);
-}
-```
----
-# Important notes
-- Use **short delays** appropriate to your bus speed; `HAL_Delay(1)` is safe but slow.
-- If the **slave keeps SDA low even after 9 clocks**, it may be latched or powered incorrectly; cycling power to the slave may be required.
-- If the **STM32 I2C peripheral itself** is wedged in BUSY, the RCC **force/reset** step is often helpful before re-init.
-- Make sure pull-ups are present on the bus.
----
-# Best practice
-In a robust design, on I2C error:
-1. Abort transfer
-2. Deinit I2C
-3. GPIO clock-pulse recovery
-4. Manual STOP
-5. Peripheral force-reset if still busy
-6. Reinit I2C
-7. Retry transaction once
-If you want, I can provide a **CubeWL-ready recovery function** using your exact I2C instance and pins.</t>
-  </si>
-  <si>
     <t>I need lower power consumption on STM32CubeWL while preserving wake-up reliability. Which low-power configuration points should be audited first (clocks, GPIO state, peripherals, wake-up sources)?</t>
   </si>
   <si>
@@ -11758,6 +8743,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -12045,7 +9034,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C97"/>
+  <dimension ref="A1:C71"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="80" customWidth="1"/>
@@ -12105,18 +9094,18 @@
         <v>11</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>12</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
@@ -12127,7 +9116,7 @@
         <v>16</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
@@ -12138,29 +9127,29 @@
         <v>18</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>19</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
@@ -12171,213 +9160,213 @@
         <v>25</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>26</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>33</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B18" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>40</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B21" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C21" s="2" t="s">
         <v>47</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B24" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C24" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B27" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C27" s="2" t="s">
         <v>61</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>68</v>
@@ -12385,10 +9374,10 @@
     </row>
     <row r="31" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>68</v>
@@ -12396,10 +9385,10 @@
     </row>
     <row r="32" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C32" s="2" t="s">
         <v>68</v>
@@ -12407,21 +9396,21 @@
     </row>
     <row r="33" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>77</v>
@@ -12429,10 +9418,10 @@
     </row>
     <row r="35" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>77</v>
@@ -12440,694 +9429,408 @@
     </row>
     <row r="36" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
     </row>
     <row r="38" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C38" s="2" t="s">
         <v>84</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="39" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
     </row>
     <row r="40" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
     </row>
     <row r="41" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C41" s="2" t="s">
         <v>91</v>
-      </c>
-      <c r="B41" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="C41" s="2" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="42" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="43" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="44" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="C44" s="2" t="s">
         <v>98</v>
-      </c>
-      <c r="B44" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="45" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="46" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="47" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C47" s="2" t="s">
         <v>105</v>
-      </c>
-      <c r="B47" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="C47" s="2" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="48" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
     </row>
     <row r="49" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
     </row>
     <row r="50" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="B50" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C50" s="2" t="s">
         <v>112</v>
-      </c>
-      <c r="C50" s="2" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="51" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
     </row>
     <row r="52" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
     </row>
     <row r="53" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="B53" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="C53" s="2" t="s">
         <v>119</v>
-      </c>
-      <c r="C53" s="2" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="54" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
     </row>
     <row r="55" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
     </row>
     <row r="56" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="B56" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="C56" s="2" t="s">
         <v>126</v>
-      </c>
-      <c r="C56" s="2" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="57" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
     </row>
     <row r="58" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="59" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A59" s="2" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
     </row>
     <row r="60" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="B60" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="C60" s="2" t="s">
         <v>135</v>
-      </c>
-      <c r="C60" s="2" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="61" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A61" s="2" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>131</v>
+        <v>142</v>
       </c>
     </row>
     <row r="62" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="63" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="B63" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="C63" s="2" t="s">
         <v>142</v>
-      </c>
-      <c r="C63" s="2" t="s">
-        <v>140</v>
       </c>
     </row>
     <row r="64" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
     </row>
     <row r="65" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
     </row>
     <row r="66" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A66" s="2" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
     </row>
     <row r="67" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
     </row>
     <row r="68" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A68" s="2" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
     </row>
     <row r="69" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>149</v>
+        <v>161</v>
       </c>
     </row>
     <row r="70" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
     </row>
     <row r="71" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="72" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A72" s="2" t="s">
         <v>161</v>
-      </c>
-      <c r="B72" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="C72" s="2" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="73" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A73" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="B73" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="C73" s="2" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="74" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A74" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="B74" s="2" t="s">
-        <v>166</v>
-      </c>
-      <c r="C74" s="2" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="75" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A75" s="2" t="s">
-        <v>168</v>
-      </c>
-      <c r="B75" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="C75" s="2" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="76" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A76" s="2" t="s">
-        <v>170</v>
-      </c>
-      <c r="B76" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="C76" s="2" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="77" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A77" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="B77" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="C77" s="2" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="78" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A78" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="B78" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="C78" s="2" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="79" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A79" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="B79" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="C79" s="2" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="80" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A80" s="2" t="s">
-        <v>179</v>
-      </c>
-      <c r="B80" s="2" t="s">
-        <v>180</v>
-      </c>
-      <c r="C80" s="2" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="81" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A81" s="2" t="s">
-        <v>181</v>
-      </c>
-      <c r="B81" s="2" t="s">
-        <v>182</v>
-      </c>
-      <c r="C81" s="2" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="82" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A82" s="2" t="s">
-        <v>183</v>
-      </c>
-      <c r="B82" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="C82" s="2" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="83" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A83" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="B83" s="2" t="s">
-        <v>187</v>
-      </c>
-      <c r="C83" s="2" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="84" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A84" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="B84" s="2" t="s">
-        <v>189</v>
-      </c>
-      <c r="C84" s="2" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="85" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A85" s="2" t="s">
-        <v>190</v>
-      </c>
-      <c r="B85" s="2" t="s">
-        <v>191</v>
-      </c>
-      <c r="C85" s="2" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="86" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A86" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="B86" s="2" t="s">
-        <v>193</v>
-      </c>
-      <c r="C86" s="2" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="87" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A87" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="B87" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="C87" s="2" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="88" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A88" s="2" t="s">
-        <v>197</v>
-      </c>
-      <c r="B88" s="2" t="s">
-        <v>198</v>
-      </c>
-      <c r="C88" s="2" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="89" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A89" s="2" t="s">
-        <v>199</v>
-      </c>
-      <c r="B89" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="C89" s="2" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="90" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A90" s="2" t="s">
-        <v>201</v>
-      </c>
-      <c r="B90" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="C90" s="2" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="91" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A91" s="2" t="s">
-        <v>204</v>
-      </c>
-      <c r="B91" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="C91" s="2" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="92" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A92" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="B92" s="2" t="s">
-        <v>207</v>
-      </c>
-      <c r="C92" s="2" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="93" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A93" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="B93" s="2" t="s">
-        <v>209</v>
-      </c>
-      <c r="C93" s="2" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="94" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A94" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="B94" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="C94" s="2" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="95" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A95" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="B95" s="2" t="s">
-        <v>214</v>
-      </c>
-      <c r="C95" s="2" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="96" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A96" s="2" t="s">
-        <v>215</v>
-      </c>
-      <c r="B96" s="2" t="s">
-        <v>216</v>
-      </c>
-      <c r="C96" s="2" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="97" spans="1:3" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A97" s="2" t="s">
-        <v>217</v>
-      </c>
-      <c r="B97" s="2" t="s">
-        <v>218</v>
-      </c>
-      <c r="C97" s="2" t="s">
-        <v>212</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C97" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:C71" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
-  <clbl:label id="{75e027c9-20d5-47d5-b82f-77d7cd041e8f}" enabled="0" method="" siteId="{75e027c9-20d5-47d5-b82f-77d7cd041e8f}" removed="1"/>
+  <clbl:label id="{cf8c7287-838c-46dd-b281-b1140229e67a}" enabled="1" method="Privileged" siteId="{75e027c9-20d5-47d5-b82f-77d7cd041e8f}" removed="0"/>
 </clbl:labelList>
 </file>
</xml_diff>